<commit_message>
Ajuste Modelo Caso de Uso
</commit_message>
<xml_diff>
--- a/AprovAI/6.Gerenciamento de Projeto/AprovAI - Planejamento e Controle do Projeto.xlsx
+++ b/AprovAI/6.Gerenciamento de Projeto/AprovAI - Planejamento e Controle do Projeto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiag\Downloads\EngenhariaSoftware_AprovAI\AprovAI\AprovAI\6.Gerenciamento de Projeto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D4818BC-0B3A-41E8-B5FE-52BF2D5F9902}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A03D902-B841-4702-BF19-88D23DCBE806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="718" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="718" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Equipe" sheetId="1" r:id="rId1"/>
@@ -6550,6 +6550,42 @@
     <xf numFmtId="164" fontId="43" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="29" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="3" borderId="1" xfId="10" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="169" fontId="29" fillId="9" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="9" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6557,17 +6593,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="22" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="7" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6577,38 +6607,17 @@
     <xf numFmtId="164" fontId="13" fillId="5" borderId="2" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="28" fillId="10" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="33" fillId="15" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6624,6 +6633,33 @@
     <xf numFmtId="164" fontId="33" fillId="15" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="32" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="28" fillId="10" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="16" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6653,42 +6689,6 @@
     </xf>
     <xf numFmtId="164" fontId="31" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="3" borderId="1" xfId="10" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="169" fontId="29" fillId="9" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="30" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="9" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="17">
@@ -6711,30 +6711,6 @@
     <cellStyle name="Result2" xfId="15" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
   </cellStyles>
   <dxfs count="10">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF8080"/>
-          <bgColor rgb="FFFF8080"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFCCFFCC"/>
-          <bgColor rgb="FFCCFFCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <b/>
@@ -6769,6 +6745,30 @@
       <font>
         <color rgb="FF666699"/>
       </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF8080"/>
+          <bgColor rgb="FFFF8080"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCCFFCC"/>
+          <bgColor rgb="FFCCFFCC"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -8580,18 +8580,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="125" t="s">
+      <c r="A1" s="134" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="125"/>
-      <c r="C1" s="125"/>
+      <c r="B1" s="134"/>
+      <c r="C1" s="134"/>
     </row>
     <row r="2" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="126" t="s">
+      <c r="A2" s="135" t="s">
         <v>218</v>
       </c>
-      <c r="B2" s="126"/>
-      <c r="C2" s="126"/>
+      <c r="B2" s="135"/>
+      <c r="C2" s="135"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -8722,19 +8722,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="134" t="s">
+      <c r="A1" s="136" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="134"/>
-      <c r="C1" s="134"/>
+      <c r="B1" s="136"/>
+      <c r="C1" s="136"/>
     </row>
     <row r="2" spans="1:5" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="135" t="s">
+      <c r="A3" s="137" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="135"/>
-      <c r="C3" s="135"/>
+      <c r="B3" s="137"/>
+      <c r="C3" s="137"/>
     </row>
     <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
@@ -8843,11 +8843,11 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="135" t="s">
+      <c r="A14" s="137" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="135"/>
-      <c r="C14" s="135"/>
+      <c r="B14" s="137"/>
+      <c r="C14" s="137"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="30" t="s">
@@ -8959,38 +8959,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="140" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="133"/>
-      <c r="C1" s="133"/>
-      <c r="D1" s="133"/>
-      <c r="F1" s="127" t="s">
+      <c r="B1" s="140"/>
+      <c r="C1" s="140"/>
+      <c r="D1" s="140"/>
+      <c r="F1" s="141" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="127"/>
-      <c r="H1" s="127"/>
-      <c r="I1" s="127"/>
-      <c r="J1" s="127"/>
-      <c r="K1" s="127"/>
-      <c r="L1" s="127"/>
+      <c r="G1" s="141"/>
+      <c r="H1" s="141"/>
+      <c r="I1" s="141"/>
+      <c r="J1" s="141"/>
+      <c r="K1" s="141"/>
+      <c r="L1" s="141"/>
     </row>
     <row r="2" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="128" t="s">
+      <c r="A2" s="142" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="128"/>
-      <c r="C2" s="128"/>
-      <c r="D2" s="128"/>
-      <c r="F2" s="129" t="s">
+      <c r="B2" s="142"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="F2" s="143" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="129"/>
-      <c r="H2" s="129"/>
-      <c r="I2" s="129"/>
-      <c r="J2" s="129"/>
-      <c r="K2" s="129"/>
-      <c r="L2" s="129"/>
+      <c r="G2" s="143"/>
+      <c r="H2" s="143"/>
+      <c r="I2" s="143"/>
+      <c r="J2" s="143"/>
+      <c r="K2" s="143"/>
+      <c r="L2" s="143"/>
     </row>
     <row r="3" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
@@ -9011,20 +9011,20 @@
       <c r="G3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="130" t="s">
+      <c r="H3" s="144" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="130"/>
-      <c r="J3" s="130"/>
-      <c r="K3" s="130"/>
-      <c r="L3" s="130"/>
+      <c r="I3" s="144"/>
+      <c r="J3" s="144"/>
+      <c r="K3" s="144"/>
+      <c r="L3" s="144"/>
     </row>
     <row r="4" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="131" t="s">
+      <c r="A4" s="138" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="131"/>
-      <c r="C4" s="131"/>
+      <c r="B4" s="138"/>
+      <c r="C4" s="138"/>
       <c r="D4" s="8" t="s">
         <v>17</v>
       </c>
@@ -9267,11 +9267,11 @@
       </c>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="131" t="s">
+      <c r="A11" s="138" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="131"/>
-      <c r="C11" s="131"/>
+      <c r="B11" s="138"/>
+      <c r="C11" s="138"/>
       <c r="D11" s="8">
         <f>SUM(D5:D10)</f>
         <v>10</v>
@@ -9534,11 +9534,11 @@
       <c r="L20" s="21"/>
     </row>
     <row r="21" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="131" t="s">
+      <c r="A21" s="138" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="131"/>
-      <c r="C21" s="131"/>
+      <c r="B21" s="138"/>
+      <c r="C21" s="138"/>
       <c r="D21" s="8">
         <f>SUM(D12:D20)</f>
         <v>82</v>
@@ -9901,11 +9901,11 @@
       </c>
     </row>
     <row r="41" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="131" t="s">
+      <c r="A41" s="138" t="s">
         <v>41</v>
       </c>
-      <c r="B41" s="131"/>
-      <c r="C41" s="131"/>
+      <c r="B41" s="138"/>
+      <c r="C41" s="138"/>
       <c r="D41" s="8">
         <f>SUM(D22:D40)</f>
         <v>130</v>
@@ -10038,9 +10038,9 @@
       </c>
     </row>
     <row r="51" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="132"/>
-      <c r="B51" s="132"/>
-      <c r="C51" s="132"/>
+      <c r="A51" s="139"/>
+      <c r="B51" s="139"/>
+      <c r="C51" s="139"/>
       <c r="D51" s="8">
         <f>SUM(D42:D50)</f>
         <v>85</v>
@@ -10054,16 +10054,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="F1:L1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="F2:L2"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="A4:C4"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A41:C41"/>
     <mergeCell ref="A51:C51"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="F1:L1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="F2:L2"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="A4:C4"/>
   </mergeCells>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="1.1437007874015752" bottom="1.1437007874015752" header="0.75000000000000011" footer="0.75000000000000011"/>
   <pageSetup paperSize="0" fitToWidth="0" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
@@ -10134,19 +10134,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="67" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="136" t="s">
+      <c r="A1" s="152" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="136"/>
-      <c r="C1" s="136"/>
-      <c r="D1" s="136"/>
-      <c r="E1" s="136"/>
-      <c r="F1" s="136"/>
-      <c r="G1" s="136"/>
-      <c r="H1" s="136"/>
-      <c r="I1" s="136"/>
-      <c r="J1" s="136"/>
-      <c r="K1" s="136"/>
+      <c r="B1" s="152"/>
+      <c r="C1" s="152"/>
+      <c r="D1" s="152"/>
+      <c r="E1" s="152"/>
+      <c r="F1" s="152"/>
+      <c r="G1" s="152"/>
+      <c r="H1" s="152"/>
+      <c r="I1" s="152"/>
+      <c r="J1" s="152"/>
+      <c r="K1" s="152"/>
     </row>
     <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
@@ -10300,10 +10300,10 @@
       </c>
     </row>
     <row r="33" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D33" s="141" t="s">
+      <c r="D33" s="153" t="s">
         <v>121</v>
       </c>
-      <c r="E33" s="141"/>
+      <c r="E33" s="153"/>
     </row>
     <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="D34" s="70">
@@ -10355,64 +10355,64 @@
     </row>
     <row r="40" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="41" spans="1:11" s="67" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="142" t="s">
+      <c r="A41" s="154" t="s">
         <v>128</v>
       </c>
-      <c r="B41" s="142"/>
-      <c r="C41" s="142"/>
-      <c r="D41" s="142"/>
-      <c r="E41" s="142"/>
-      <c r="F41" s="142"/>
-      <c r="G41" s="142"/>
-      <c r="H41" s="142"/>
-      <c r="I41" s="142"/>
-      <c r="J41" s="142"/>
-      <c r="K41" s="142"/>
+      <c r="B41" s="154"/>
+      <c r="C41" s="154"/>
+      <c r="D41" s="154"/>
+      <c r="E41" s="154"/>
+      <c r="F41" s="154"/>
+      <c r="G41" s="154"/>
+      <c r="H41" s="154"/>
+      <c r="I41" s="154"/>
+      <c r="J41" s="154"/>
+      <c r="K41" s="154"/>
     </row>
     <row r="42" spans="1:11" s="67" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="143" t="s">
+      <c r="A42" s="155" t="s">
         <v>129</v>
       </c>
-      <c r="B42" s="143"/>
-      <c r="C42" s="143"/>
-      <c r="D42" s="143"/>
-      <c r="E42" s="143"/>
-      <c r="F42" s="143"/>
-      <c r="G42" s="143"/>
-      <c r="H42" s="143"/>
-      <c r="I42" s="143"/>
-      <c r="J42" s="143"/>
-      <c r="K42" s="143"/>
+      <c r="B42" s="155"/>
+      <c r="C42" s="155"/>
+      <c r="D42" s="155"/>
+      <c r="E42" s="155"/>
+      <c r="F42" s="155"/>
+      <c r="G42" s="155"/>
+      <c r="H42" s="155"/>
+      <c r="I42" s="155"/>
+      <c r="J42" s="155"/>
+      <c r="K42" s="155"/>
     </row>
     <row r="43" spans="1:11" s="67" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="144" t="s">
+      <c r="A43" s="156" t="s">
         <v>130</v>
       </c>
-      <c r="B43" s="144"/>
-      <c r="C43" s="144"/>
-      <c r="D43" s="144"/>
-      <c r="E43" s="144"/>
-      <c r="F43" s="144"/>
-      <c r="G43" s="144"/>
-      <c r="H43" s="144"/>
-      <c r="I43" s="144"/>
-      <c r="J43" s="144"/>
-      <c r="K43" s="144"/>
+      <c r="B43" s="156"/>
+      <c r="C43" s="156"/>
+      <c r="D43" s="156"/>
+      <c r="E43" s="156"/>
+      <c r="F43" s="156"/>
+      <c r="G43" s="156"/>
+      <c r="H43" s="156"/>
+      <c r="I43" s="156"/>
+      <c r="J43" s="156"/>
+      <c r="K43" s="156"/>
     </row>
     <row r="44" spans="1:11" s="67" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="140" t="s">
+      <c r="A44" s="151" t="s">
         <v>131</v>
       </c>
-      <c r="B44" s="140"/>
-      <c r="C44" s="140"/>
-      <c r="D44" s="140"/>
-      <c r="E44" s="140"/>
-      <c r="F44" s="140"/>
-      <c r="G44" s="140"/>
-      <c r="H44" s="140"/>
-      <c r="I44" s="140"/>
-      <c r="J44" s="140"/>
-      <c r="K44" s="140"/>
+      <c r="B44" s="151"/>
+      <c r="C44" s="151"/>
+      <c r="D44" s="151"/>
+      <c r="E44" s="151"/>
+      <c r="F44" s="151"/>
+      <c r="G44" s="151"/>
+      <c r="H44" s="151"/>
+      <c r="I44" s="151"/>
+      <c r="J44" s="151"/>
+      <c r="K44" s="151"/>
     </row>
     <row r="45" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="46" spans="1:11" ht="15" x14ac:dyDescent="0.25">
@@ -10685,6 +10685,12 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A43:K43"/>
     <mergeCell ref="H49:I49"/>
     <mergeCell ref="H50:I50"/>
     <mergeCell ref="H59:I59"/>
@@ -10699,21 +10705,15 @@
     <mergeCell ref="F48:F49"/>
     <mergeCell ref="G48:G49"/>
     <mergeCell ref="H48:K48"/>
-    <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A42:K42"/>
-    <mergeCell ref="A43:K43"/>
   </mergeCells>
   <conditionalFormatting sqref="F50:F60">
-    <cfRule type="cellIs" dxfId="2" priority="8" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="8" stopIfTrue="1" operator="equal">
       <formula>$D$15</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="9" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="9" stopIfTrue="1" operator="equal">
       <formula>$D$16</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="10" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="10" stopIfTrue="1" operator="equal">
       <formula>$D$17</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10755,54 +10755,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="136" t="s">
+      <c r="A1" s="152" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="136"/>
-      <c r="C1" s="136"/>
-      <c r="D1" s="136"/>
-      <c r="E1" s="136"/>
-      <c r="F1" s="136"/>
-      <c r="G1" s="136"/>
-      <c r="H1" s="136"/>
-      <c r="I1" s="136"/>
-      <c r="J1" s="136"/>
-      <c r="K1" s="136"/>
+      <c r="B1" s="152"/>
+      <c r="C1" s="152"/>
+      <c r="D1" s="152"/>
+      <c r="E1" s="152"/>
+      <c r="F1" s="152"/>
+      <c r="G1" s="152"/>
+      <c r="H1" s="152"/>
+      <c r="I1" s="152"/>
+      <c r="J1" s="152"/>
+      <c r="K1" s="152"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="137" t="s">
+      <c r="A2" s="157" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="137"/>
-      <c r="C2" s="137"/>
-      <c r="D2" s="137"/>
+      <c r="B2" s="157"/>
+      <c r="C2" s="157"/>
+      <c r="D2" s="157"/>
       <c r="E2" s="44">
         <f>Planejamento!$B$10</f>
         <v>429.8</v>
       </c>
       <c r="F2" s="45"/>
-      <c r="G2" s="137" t="s">
+      <c r="G2" s="157" t="s">
         <v>76</v>
       </c>
-      <c r="H2" s="137"/>
-      <c r="I2" s="137"/>
-      <c r="J2" s="137"/>
+      <c r="H2" s="157"/>
+      <c r="I2" s="157"/>
+      <c r="J2" s="157"/>
       <c r="K2" s="44"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="46"/>
       <c r="B3" s="47"/>
-      <c r="C3" s="138" t="s">
+      <c r="C3" s="158" t="s">
         <v>77</v>
       </c>
-      <c r="D3" s="138"/>
-      <c r="E3" s="138"/>
+      <c r="D3" s="158"/>
+      <c r="E3" s="158"/>
       <c r="F3" s="48"/>
-      <c r="G3" s="139" t="s">
+      <c r="G3" s="159" t="s">
         <v>78</v>
       </c>
-      <c r="H3" s="139"/>
-      <c r="I3" s="139"/>
+      <c r="H3" s="159"/>
+      <c r="I3" s="159"/>
       <c r="J3" s="50"/>
       <c r="K3" s="51"/>
     </row>
@@ -10845,23 +10845,23 @@
       <c r="A5" s="53">
         <v>1</v>
       </c>
-      <c r="B5" s="161" t="s">
+      <c r="B5" s="125" t="s">
         <v>87</v>
       </c>
-      <c r="C5" s="163">
+      <c r="C5" s="127">
         <v>46099</v>
       </c>
-      <c r="D5" s="163">
+      <c r="D5" s="127">
         <v>46113</v>
       </c>
       <c r="E5" s="54">
         <v>12</v>
       </c>
-      <c r="F5" s="164" t="s">
+      <c r="F5" s="128" t="s">
         <v>88</v>
       </c>
-      <c r="G5" s="163"/>
-      <c r="H5" s="163"/>
+      <c r="G5" s="127"/>
+      <c r="H5" s="127"/>
       <c r="I5" s="54">
         <v>8</v>
       </c>
@@ -10869,7 +10869,7 @@
         <f>E5-I5</f>
         <v>4</v>
       </c>
-      <c r="K5" s="165" t="s">
+      <c r="K5" s="129" t="s">
         <v>222</v>
       </c>
     </row>
@@ -10877,26 +10877,26 @@
       <c r="A6" s="53">
         <v>2</v>
       </c>
-      <c r="B6" s="162" t="s">
+      <c r="B6" s="126" t="s">
         <v>252</v>
       </c>
-      <c r="C6" s="163">
+      <c r="C6" s="127">
         <v>46113</v>
       </c>
-      <c r="D6" s="163">
+      <c r="D6" s="127">
         <v>46127</v>
       </c>
       <c r="E6" s="54">
         <v>16</v>
       </c>
-      <c r="F6" s="164" t="s">
+      <c r="F6" s="128" t="s">
         <v>89</v>
       </c>
-      <c r="G6" s="163"/>
-      <c r="H6" s="163"/>
+      <c r="G6" s="127"/>
+      <c r="H6" s="127"/>
       <c r="I6" s="56"/>
       <c r="J6" s="57"/>
-      <c r="K6" s="165" t="s">
+      <c r="K6" s="129" t="s">
         <v>222</v>
       </c>
     </row>
@@ -10904,26 +10904,26 @@
       <c r="A7" s="53">
         <v>3</v>
       </c>
-      <c r="B7" s="162" t="s">
+      <c r="B7" s="126" t="s">
         <v>224</v>
       </c>
-      <c r="C7" s="163">
+      <c r="C7" s="127">
         <v>46127</v>
       </c>
-      <c r="D7" s="163">
+      <c r="D7" s="127">
         <v>46141</v>
       </c>
       <c r="E7" s="54">
         <v>23</v>
       </c>
-      <c r="F7" s="164" t="s">
+      <c r="F7" s="128" t="s">
         <v>89</v>
       </c>
-      <c r="G7" s="163"/>
-      <c r="H7" s="163"/>
+      <c r="G7" s="127"/>
+      <c r="H7" s="127"/>
       <c r="I7" s="56"/>
       <c r="J7" s="57"/>
-      <c r="K7" s="165" t="s">
+      <c r="K7" s="129" t="s">
         <v>222</v>
       </c>
     </row>
@@ -10931,26 +10931,26 @@
       <c r="A8" s="53">
         <v>4</v>
       </c>
-      <c r="B8" s="162" t="s">
+      <c r="B8" s="126" t="s">
         <v>253</v>
       </c>
-      <c r="C8" s="163">
+      <c r="C8" s="127">
         <v>46141</v>
       </c>
-      <c r="D8" s="163">
+      <c r="D8" s="127">
         <v>46155</v>
       </c>
       <c r="E8" s="54">
         <v>23</v>
       </c>
-      <c r="F8" s="164" t="s">
+      <c r="F8" s="128" t="s">
         <v>89</v>
       </c>
-      <c r="G8" s="166"/>
-      <c r="H8" s="166"/>
+      <c r="G8" s="130"/>
+      <c r="H8" s="130"/>
       <c r="I8" s="58"/>
       <c r="J8" s="59"/>
-      <c r="K8" s="165" t="s">
+      <c r="K8" s="129" t="s">
         <v>222</v>
       </c>
     </row>
@@ -10958,26 +10958,26 @@
       <c r="A9" s="53">
         <v>5</v>
       </c>
-      <c r="B9" s="162" t="s">
+      <c r="B9" s="126" t="s">
         <v>255</v>
       </c>
-      <c r="C9" s="163">
+      <c r="C9" s="127">
         <v>46155</v>
       </c>
-      <c r="D9" s="163">
+      <c r="D9" s="127">
         <v>46169</v>
       </c>
       <c r="E9" s="54">
         <v>16</v>
       </c>
-      <c r="F9" s="164" t="s">
+      <c r="F9" s="128" t="s">
         <v>89</v>
       </c>
-      <c r="G9" s="166"/>
-      <c r="H9" s="166"/>
+      <c r="G9" s="130"/>
+      <c r="H9" s="130"/>
       <c r="I9" s="58"/>
       <c r="J9" s="59"/>
-      <c r="K9" s="165" t="s">
+      <c r="K9" s="129" t="s">
         <v>222</v>
       </c>
     </row>
@@ -10985,26 +10985,26 @@
       <c r="A10" s="53">
         <v>6</v>
       </c>
-      <c r="B10" s="162" t="s">
+      <c r="B10" s="126" t="s">
         <v>256</v>
       </c>
-      <c r="C10" s="163">
+      <c r="C10" s="127">
         <v>46169</v>
       </c>
-      <c r="D10" s="163">
+      <c r="D10" s="127">
         <v>46183</v>
       </c>
       <c r="E10" s="54">
         <v>24</v>
       </c>
-      <c r="F10" s="164" t="s">
+      <c r="F10" s="128" t="s">
         <v>89</v>
       </c>
-      <c r="G10" s="166"/>
-      <c r="H10" s="166"/>
+      <c r="G10" s="130"/>
+      <c r="H10" s="130"/>
       <c r="I10" s="58"/>
       <c r="J10" s="59"/>
-      <c r="K10" s="165" t="s">
+      <c r="K10" s="129" t="s">
         <v>222</v>
       </c>
     </row>
@@ -11012,61 +11012,61 @@
       <c r="A11" s="53">
         <v>7</v>
       </c>
-      <c r="B11" s="162"/>
-      <c r="C11" s="163"/>
-      <c r="D11" s="163"/>
+      <c r="B11" s="126"/>
+      <c r="C11" s="127"/>
+      <c r="D11" s="127"/>
       <c r="E11" s="54"/>
-      <c r="F11" s="164"/>
-      <c r="G11" s="166"/>
-      <c r="H11" s="166"/>
+      <c r="F11" s="128"/>
+      <c r="G11" s="130"/>
+      <c r="H11" s="130"/>
       <c r="I11" s="58"/>
       <c r="J11" s="59"/>
-      <c r="K11" s="165"/>
+      <c r="K11" s="129"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="53">
         <v>8</v>
       </c>
-      <c r="B12" s="167"/>
-      <c r="C12" s="166"/>
-      <c r="D12" s="166"/>
+      <c r="B12" s="131"/>
+      <c r="C12" s="130"/>
+      <c r="D12" s="130"/>
       <c r="E12" s="54"/>
-      <c r="F12" s="168"/>
-      <c r="G12" s="166"/>
-      <c r="H12" s="166"/>
+      <c r="F12" s="132"/>
+      <c r="G12" s="130"/>
+      <c r="H12" s="130"/>
       <c r="I12" s="58"/>
       <c r="J12" s="59"/>
-      <c r="K12" s="169"/>
+      <c r="K12" s="133"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="53">
         <v>9</v>
       </c>
-      <c r="B13" s="167"/>
-      <c r="C13" s="166"/>
-      <c r="D13" s="166"/>
+      <c r="B13" s="131"/>
+      <c r="C13" s="130"/>
+      <c r="D13" s="130"/>
       <c r="E13" s="54"/>
-      <c r="F13" s="168"/>
-      <c r="G13" s="166"/>
-      <c r="H13" s="166"/>
+      <c r="F13" s="132"/>
+      <c r="G13" s="130"/>
+      <c r="H13" s="130"/>
       <c r="I13" s="58"/>
       <c r="J13" s="59"/>
-      <c r="K13" s="169"/>
+      <c r="K13" s="133"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="53">
         <v>10</v>
       </c>
-      <c r="B14" s="167"/>
-      <c r="C14" s="166"/>
-      <c r="D14" s="166"/>
+      <c r="B14" s="131"/>
+      <c r="C14" s="130"/>
+      <c r="D14" s="130"/>
       <c r="E14" s="54"/>
-      <c r="F14" s="168"/>
-      <c r="G14" s="166"/>
-      <c r="H14" s="166"/>
+      <c r="F14" s="132"/>
+      <c r="G14" s="130"/>
+      <c r="H14" s="130"/>
       <c r="I14" s="58"/>
       <c r="J14" s="59"/>
-      <c r="K14" s="169"/>
+      <c r="K14" s="133"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="60"/>
@@ -11102,29 +11102,29 @@
     <mergeCell ref="G3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:D14">
-    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="6" stopIfTrue="1">
       <formula>OR($F5="Planned",$F5="Unplanned")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="7" stopIfTrue="1">
       <formula>$F5="Ongoing"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5:F14">
-    <cfRule type="expression" dxfId="7" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="1" stopIfTrue="1">
       <formula>$F5="Planned"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="2" stopIfTrue="1">
       <formula>$F5="Ongoing"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="3" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="3" stopIfTrue="1" operator="equal">
       <formula>"Unplanned"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:H14">
-    <cfRule type="expression" dxfId="4" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="1" priority="4" stopIfTrue="1">
       <formula>OR($F5="Planned",$F5="Unplanned")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="5" stopIfTrue="1">
       <formula>$F5="Ongoing"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11163,116 +11163,116 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" s="67" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="153" t="s">
+      <c r="A1" s="162" t="s">
         <v>144</v>
       </c>
-      <c r="B1" s="153"/>
-      <c r="C1" s="153"/>
-      <c r="D1" s="153"/>
-      <c r="E1" s="153"/>
-      <c r="F1" s="153"/>
-      <c r="G1" s="153"/>
-      <c r="H1" s="153"/>
-      <c r="I1" s="153"/>
-      <c r="J1" s="153"/>
-      <c r="K1" s="153"/>
-      <c r="L1" s="153"/>
-      <c r="M1" s="153"/>
-      <c r="N1" s="153"/>
+      <c r="B1" s="162"/>
+      <c r="C1" s="162"/>
+      <c r="D1" s="162"/>
+      <c r="E1" s="162"/>
+      <c r="F1" s="162"/>
+      <c r="G1" s="162"/>
+      <c r="H1" s="162"/>
+      <c r="I1" s="162"/>
+      <c r="J1" s="162"/>
+      <c r="K1" s="162"/>
+      <c r="L1" s="162"/>
+      <c r="M1" s="162"/>
+      <c r="N1" s="162"/>
     </row>
     <row r="2" spans="1:23" s="87" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="154" t="s">
+      <c r="A2" s="163" t="s">
         <v>128</v>
       </c>
-      <c r="B2" s="154"/>
-      <c r="C2" s="154"/>
-      <c r="D2" s="154"/>
-      <c r="E2" s="154"/>
-      <c r="F2" s="154"/>
-      <c r="G2" s="154"/>
-      <c r="H2" s="154"/>
-      <c r="I2" s="154"/>
-      <c r="J2" s="154"/>
-      <c r="K2" s="154"/>
-      <c r="L2" s="154"/>
-      <c r="M2" s="154"/>
-      <c r="N2" s="154"/>
+      <c r="B2" s="163"/>
+      <c r="C2" s="163"/>
+      <c r="D2" s="163"/>
+      <c r="E2" s="163"/>
+      <c r="F2" s="163"/>
+      <c r="G2" s="163"/>
+      <c r="H2" s="163"/>
+      <c r="I2" s="163"/>
+      <c r="J2" s="163"/>
+      <c r="K2" s="163"/>
+      <c r="L2" s="163"/>
+      <c r="M2" s="163"/>
+      <c r="N2" s="163"/>
     </row>
     <row r="3" spans="1:23" s="87" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="155" t="s">
+      <c r="A3" s="164" t="s">
         <v>145</v>
       </c>
-      <c r="B3" s="155"/>
-      <c r="C3" s="155"/>
-      <c r="D3" s="155"/>
-      <c r="E3" s="155"/>
-      <c r="F3" s="155"/>
-      <c r="G3" s="155"/>
-      <c r="H3" s="155"/>
-      <c r="I3" s="155"/>
-      <c r="J3" s="155"/>
-      <c r="K3" s="155"/>
-      <c r="L3" s="155"/>
-      <c r="M3" s="155"/>
-      <c r="N3" s="155"/>
+      <c r="B3" s="164"/>
+      <c r="C3" s="164"/>
+      <c r="D3" s="164"/>
+      <c r="E3" s="164"/>
+      <c r="F3" s="164"/>
+      <c r="G3" s="164"/>
+      <c r="H3" s="164"/>
+      <c r="I3" s="164"/>
+      <c r="J3" s="164"/>
+      <c r="K3" s="164"/>
+      <c r="L3" s="164"/>
+      <c r="M3" s="164"/>
+      <c r="N3" s="164"/>
     </row>
     <row r="4" spans="1:23" s="87" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="156" t="s">
+      <c r="A4" s="165" t="s">
         <v>146</v>
       </c>
-      <c r="B4" s="156"/>
-      <c r="C4" s="156"/>
-      <c r="D4" s="156"/>
-      <c r="E4" s="156"/>
-      <c r="F4" s="156"/>
-      <c r="G4" s="156"/>
-      <c r="H4" s="156"/>
-      <c r="I4" s="156"/>
-      <c r="J4" s="156"/>
-      <c r="K4" s="156"/>
-      <c r="L4" s="156"/>
-      <c r="M4" s="156"/>
-      <c r="N4" s="156"/>
+      <c r="B4" s="165"/>
+      <c r="C4" s="165"/>
+      <c r="D4" s="165"/>
+      <c r="E4" s="165"/>
+      <c r="F4" s="165"/>
+      <c r="G4" s="165"/>
+      <c r="H4" s="165"/>
+      <c r="I4" s="165"/>
+      <c r="J4" s="165"/>
+      <c r="K4" s="165"/>
+      <c r="L4" s="165"/>
+      <c r="M4" s="165"/>
+      <c r="N4" s="165"/>
     </row>
     <row r="5" spans="1:23" s="87" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="157" t="s">
+      <c r="A5" s="166" t="s">
         <v>147</v>
       </c>
-      <c r="B5" s="157"/>
-      <c r="C5" s="157"/>
-      <c r="D5" s="157"/>
-      <c r="E5" s="157"/>
-      <c r="F5" s="157"/>
-      <c r="G5" s="157"/>
-      <c r="H5" s="157"/>
-      <c r="I5" s="157"/>
-      <c r="J5" s="157"/>
-      <c r="K5" s="157"/>
-      <c r="L5" s="157"/>
-      <c r="M5" s="157"/>
-      <c r="N5" s="157"/>
+      <c r="B5" s="166"/>
+      <c r="C5" s="166"/>
+      <c r="D5" s="166"/>
+      <c r="E5" s="166"/>
+      <c r="F5" s="166"/>
+      <c r="G5" s="166"/>
+      <c r="H5" s="166"/>
+      <c r="I5" s="166"/>
+      <c r="J5" s="166"/>
+      <c r="K5" s="166"/>
+      <c r="L5" s="166"/>
+      <c r="M5" s="166"/>
+      <c r="N5" s="166"/>
     </row>
     <row r="6" spans="1:23" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="7" spans="1:23" s="4" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="151" t="s">
+      <c r="A7" s="160" t="s">
         <v>148</v>
       </c>
-      <c r="B7" s="151"/>
-      <c r="D7" s="151" t="s">
+      <c r="B7" s="160"/>
+      <c r="D7" s="160" t="s">
         <v>149</v>
       </c>
-      <c r="E7" s="151"/>
-      <c r="G7" s="151" t="s">
+      <c r="E7" s="160"/>
+      <c r="G7" s="160" t="s">
         <v>150</v>
       </c>
-      <c r="H7" s="151"/>
-      <c r="I7" s="151"/>
-      <c r="J7" s="151"/>
-      <c r="K7" s="151"/>
-      <c r="M7" s="151" t="s">
+      <c r="H7" s="160"/>
+      <c r="I7" s="160"/>
+      <c r="J7" s="160"/>
+      <c r="K7" s="160"/>
+      <c r="M7" s="160" t="s">
         <v>151</v>
       </c>
-      <c r="N7" s="151"/>
+      <c r="N7" s="160"/>
     </row>
     <row r="8" spans="1:23" s="4" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="90" t="s">
@@ -11372,13 +11372,13 @@
       <c r="B11" s="89"/>
       <c r="D11" s="88"/>
       <c r="E11" s="89"/>
-      <c r="G11" s="151" t="s">
+      <c r="G11" s="160" t="s">
         <v>168</v>
       </c>
-      <c r="H11" s="151"/>
-      <c r="I11" s="151"/>
-      <c r="J11" s="151"/>
-      <c r="K11" s="151"/>
+      <c r="H11" s="160"/>
+      <c r="I11" s="160"/>
+      <c r="J11" s="160"/>
+      <c r="K11" s="160"/>
       <c r="M11" s="92" t="s">
         <v>169</v>
       </c>
@@ -11481,12 +11481,12 @@
       <c r="B16" s="89"/>
       <c r="D16" s="88"/>
       <c r="E16" s="89"/>
-      <c r="G16" s="152" t="s">
+      <c r="G16" s="161" t="s">
         <v>178</v>
       </c>
-      <c r="H16" s="152"/>
-      <c r="I16" s="152"/>
-      <c r="J16" s="152"/>
+      <c r="H16" s="161"/>
+      <c r="I16" s="161"/>
+      <c r="J16" s="161"/>
       <c r="K16" s="94">
         <f>SUM(K9,K10,K13,K14,K15)</f>
         <v>14</v>
@@ -11646,42 +11646,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="153" t="s">
+      <c r="A1" s="162" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="153"/>
-      <c r="C1" s="153"/>
-      <c r="D1" s="153"/>
-      <c r="E1" s="153"/>
-      <c r="F1" s="153"/>
-      <c r="G1" s="153"/>
-      <c r="H1" s="153"/>
-      <c r="I1" s="153"/>
-      <c r="J1" s="153"/>
-      <c r="K1" s="153"/>
-      <c r="L1" s="153"/>
-      <c r="M1" s="153"/>
-      <c r="N1" s="153"/>
+      <c r="B1" s="162"/>
+      <c r="C1" s="162"/>
+      <c r="D1" s="162"/>
+      <c r="E1" s="162"/>
+      <c r="F1" s="162"/>
+      <c r="G1" s="162"/>
+      <c r="H1" s="162"/>
+      <c r="I1" s="162"/>
+      <c r="J1" s="162"/>
+      <c r="K1" s="162"/>
+      <c r="L1" s="162"/>
+      <c r="M1" s="162"/>
+      <c r="N1" s="162"/>
     </row>
     <row r="2" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="159" t="s">
+      <c r="A3" s="168" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="159"/>
-      <c r="C3" s="159"/>
-      <c r="E3" s="159" t="s">
+      <c r="B3" s="168"/>
+      <c r="C3" s="168"/>
+      <c r="E3" s="168" t="s">
         <v>191</v>
       </c>
-      <c r="F3" s="159"/>
-      <c r="G3" s="159"/>
-      <c r="H3" s="159"/>
-      <c r="I3" s="159"/>
-      <c r="J3" s="159"/>
-      <c r="K3" s="159"/>
-      <c r="L3" s="159"/>
-      <c r="M3" s="159"/>
-      <c r="N3" s="159"/>
+      <c r="F3" s="168"/>
+      <c r="G3" s="168"/>
+      <c r="H3" s="168"/>
+      <c r="I3" s="168"/>
+      <c r="J3" s="168"/>
+      <c r="K3" s="168"/>
+      <c r="L3" s="168"/>
+      <c r="M3" s="168"/>
+      <c r="N3" s="168"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="101" t="s">
@@ -11694,25 +11694,25 @@
       <c r="C4" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="E4" s="160" t="s">
+      <c r="E4" s="169" t="s">
         <v>193</v>
       </c>
-      <c r="F4" s="158" t="s">
+      <c r="F4" s="167" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="158"/>
-      <c r="H4" s="158" t="s">
+      <c r="G4" s="167"/>
+      <c r="H4" s="167" t="s">
         <v>31</v>
       </c>
-      <c r="I4" s="158"/>
-      <c r="J4" s="158" t="s">
+      <c r="I4" s="167"/>
+      <c r="J4" s="167" t="s">
         <v>40</v>
       </c>
-      <c r="K4" s="158"/>
-      <c r="L4" s="158" t="s">
+      <c r="K4" s="167"/>
+      <c r="L4" s="167" t="s">
         <v>41</v>
       </c>
-      <c r="M4" s="158"/>
+      <c r="M4" s="167"/>
       <c r="N4" s="103"/>
     </row>
     <row r="5" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
@@ -11725,23 +11725,23 @@
       <c r="C5" s="38" t="s">
         <v>194</v>
       </c>
-      <c r="E5" s="160"/>
-      <c r="F5" s="158" t="s">
+      <c r="E5" s="169"/>
+      <c r="F5" s="167" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="158"/>
-      <c r="H5" s="158" t="s">
+      <c r="G5" s="167"/>
+      <c r="H5" s="167" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="158"/>
-      <c r="J5" s="158" t="s">
+      <c r="I5" s="167"/>
+      <c r="J5" s="167" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="158"/>
-      <c r="L5" s="158" t="s">
+      <c r="K5" s="167"/>
+      <c r="L5" s="167" t="s">
         <v>17</v>
       </c>
-      <c r="M5" s="158"/>
+      <c r="M5" s="167"/>
       <c r="N5" s="41" t="s">
         <v>195</v>
       </c>
@@ -11757,7 +11757,7 @@
       <c r="C6" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="E6" s="160"/>
+      <c r="E6" s="169"/>
       <c r="F6" s="106">
         <f>B6*G6</f>
         <v>8.6450000000000014</v>
@@ -12189,11 +12189,11 @@
       <c r="N15" s="113"/>
     </row>
     <row r="16" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A16" s="159" t="s">
+      <c r="A16" s="168" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="159"/>
-      <c r="C16" s="159"/>
+      <c r="B16" s="168"/>
+      <c r="C16" s="168"/>
       <c r="E16" s="41" t="s">
         <v>215</v>
       </c>

</xml_diff>

<commit_message>
Ajuste das Definições Modelo caso de Uso e Mapeamento de Riscos
</commit_message>
<xml_diff>
--- a/AprovAI/6.Gerenciamento de Projeto/AprovAI - Planejamento e Controle do Projeto.xlsx
+++ b/AprovAI/6.Gerenciamento de Projeto/AprovAI - Planejamento e Controle do Projeto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiag\Downloads\EngenhariaSoftware_AprovAI\AprovAI\AprovAI\6.Gerenciamento de Projeto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A03D902-B841-4702-BF19-88D23DCBE806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C570234F-919A-4612-A104-99A7C6924213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="718" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="718" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Equipe" sheetId="1" r:id="rId1"/>
@@ -4738,7 +4738,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="275">
   <si>
     <t>Equipe</t>
   </si>
@@ -5619,6 +5619,60 @@
   </si>
   <si>
     <t>UC 06 - CONSULTAR PROGRESSO, UC 07 - ACOMPANHAR DESEMPENHO, UC 09 - CONSULTAR CONTEÚDO</t>
+  </si>
+  <si>
+    <t>Indisponibilidade dos usuários para fornecer ou validar requisitos</t>
+  </si>
+  <si>
+    <t>Dificuldade em definir corretamente os requisitos devido à variedade de perfis</t>
+  </si>
+  <si>
+    <t>Limitações técnicas no desenvolvimento de funcionalidades com Inteligência Artificial</t>
+  </si>
+  <si>
+    <t>Possíveis falhas na integração entre os módulos do sistema</t>
+  </si>
+  <si>
+    <t>Baixa adesão dos usuários ao sistema após a implementação</t>
+  </si>
+  <si>
+    <t>Problemas relacionados à qualidade ou confiabilidade das recomendações da IA</t>
+  </si>
+  <si>
+    <t>Falta de experiência da equipe com determinadas tecnologias</t>
+  </si>
+  <si>
+    <t>Mudanças nos requisitos ao longo do desenvolvimen</t>
+  </si>
+  <si>
+    <t>Limitações de infraestrutura (hardware, internet, etc.)</t>
+  </si>
+  <si>
+    <t>1 - Designar um usuário chave para validação do sistema</t>
+  </si>
+  <si>
+    <t>1 - Priorizar o desenvolvimento com maior volume de usuários e tratar as especificidades dos outros perfis em versões posteriores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1- simplificar a lógica para algoritmos convencionais </t>
+  </si>
+  <si>
+    <t>1- Isolar módulos próblemáticos para que sejam tratados enquanto o sistema seja operado enquanto o erro for sendo corrigido</t>
+  </si>
+  <si>
+    <t>1- Lançar uma campanha interna de engajamento, treinamentos rápidos em vídeo e suporte dedicado para reduzir a curva de aprendizado.</t>
+  </si>
+  <si>
+    <t>1 - Adicionar um aviso de "beta" na interface e incluir um botão para o usuário reportar erros na recomendação, permitindo ajuste manual.</t>
+  </si>
+  <si>
+    <t>1 - Contratar uma consultoria externa ou profissional especialista para mentorias pontuais nos módulos mais críticos.</t>
+  </si>
+  <si>
+    <t>1 - Aplicar um processo formal de "Controle de Mudança", onde cada alteração nova gera um ajuste automático no prazo de entrega.</t>
+  </si>
+  <si>
+    <t>1 - Implementar cache local ou modo offline para as funcionalidades básicas, permitindo que o usuário trabalhe mesmo com instabilidade de rede.</t>
   </si>
 </sst>
 </file>
@@ -6599,6 +6653,18 @@
     <xf numFmtId="164" fontId="22" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="16" fillId="7" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -6607,17 +6673,23 @@
     <xf numFmtId="164" fontId="13" fillId="5" borderId="2" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="32" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="33" fillId="15" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6632,24 +6704,6 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="33" fillId="15" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="22" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
@@ -8959,38 +9013,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="140" t="s">
+      <c r="A1" s="144" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="140"/>
-      <c r="C1" s="140"/>
-      <c r="D1" s="140"/>
-      <c r="F1" s="141" t="s">
+      <c r="B1" s="144"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="F1" s="138" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="141"/>
-      <c r="H1" s="141"/>
-      <c r="I1" s="141"/>
-      <c r="J1" s="141"/>
-      <c r="K1" s="141"/>
-      <c r="L1" s="141"/>
+      <c r="G1" s="138"/>
+      <c r="H1" s="138"/>
+      <c r="I1" s="138"/>
+      <c r="J1" s="138"/>
+      <c r="K1" s="138"/>
+      <c r="L1" s="138"/>
     </row>
     <row r="2" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="142" t="s">
+      <c r="A2" s="139" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="142"/>
-      <c r="C2" s="142"/>
-      <c r="D2" s="142"/>
-      <c r="F2" s="143" t="s">
+      <c r="B2" s="139"/>
+      <c r="C2" s="139"/>
+      <c r="D2" s="139"/>
+      <c r="F2" s="140" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="143"/>
-      <c r="H2" s="143"/>
-      <c r="I2" s="143"/>
-      <c r="J2" s="143"/>
-      <c r="K2" s="143"/>
-      <c r="L2" s="143"/>
+      <c r="G2" s="140"/>
+      <c r="H2" s="140"/>
+      <c r="I2" s="140"/>
+      <c r="J2" s="140"/>
+      <c r="K2" s="140"/>
+      <c r="L2" s="140"/>
     </row>
     <row r="3" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
@@ -9011,20 +9065,20 @@
       <c r="G3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="144" t="s">
+      <c r="H3" s="141" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="144"/>
-      <c r="J3" s="144"/>
-      <c r="K3" s="144"/>
-      <c r="L3" s="144"/>
+      <c r="I3" s="141"/>
+      <c r="J3" s="141"/>
+      <c r="K3" s="141"/>
+      <c r="L3" s="141"/>
     </row>
     <row r="4" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="138" t="s">
+      <c r="A4" s="142" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="138"/>
-      <c r="C4" s="138"/>
+      <c r="B4" s="142"/>
+      <c r="C4" s="142"/>
       <c r="D4" s="8" t="s">
         <v>17</v>
       </c>
@@ -9267,11 +9321,11 @@
       </c>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="138" t="s">
+      <c r="A11" s="142" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="138"/>
-      <c r="C11" s="138"/>
+      <c r="B11" s="142"/>
+      <c r="C11" s="142"/>
       <c r="D11" s="8">
         <f>SUM(D5:D10)</f>
         <v>10</v>
@@ -9534,11 +9588,11 @@
       <c r="L20" s="21"/>
     </row>
     <row r="21" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="138" t="s">
+      <c r="A21" s="142" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="138"/>
-      <c r="C21" s="138"/>
+      <c r="B21" s="142"/>
+      <c r="C21" s="142"/>
       <c r="D21" s="8">
         <f>SUM(D12:D20)</f>
         <v>82</v>
@@ -9901,11 +9955,11 @@
       </c>
     </row>
     <row r="41" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="138" t="s">
+      <c r="A41" s="142" t="s">
         <v>41</v>
       </c>
-      <c r="B41" s="138"/>
-      <c r="C41" s="138"/>
+      <c r="B41" s="142"/>
+      <c r="C41" s="142"/>
       <c r="D41" s="8">
         <f>SUM(D22:D40)</f>
         <v>130</v>
@@ -10038,9 +10092,9 @@
       </c>
     </row>
     <row r="51" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="139"/>
-      <c r="B51" s="139"/>
-      <c r="C51" s="139"/>
+      <c r="A51" s="143"/>
+      <c r="B51" s="143"/>
+      <c r="C51" s="143"/>
       <c r="D51" s="8">
         <f>SUM(D42:D50)</f>
         <v>85</v>
@@ -10054,16 +10108,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="F1:L1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="F2:L2"/>
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="1.1437007874015752" bottom="1.1437007874015752" header="0.75000000000000011" footer="0.75000000000000011"/>
   <pageSetup paperSize="0" fitToWidth="0" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
@@ -10134,19 +10188,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="67" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="152" t="s">
+      <c r="A1" s="146" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="152"/>
-      <c r="C1" s="152"/>
-      <c r="D1" s="152"/>
-      <c r="E1" s="152"/>
-      <c r="F1" s="152"/>
-      <c r="G1" s="152"/>
-      <c r="H1" s="152"/>
-      <c r="I1" s="152"/>
-      <c r="J1" s="152"/>
-      <c r="K1" s="152"/>
+      <c r="B1" s="146"/>
+      <c r="C1" s="146"/>
+      <c r="D1" s="146"/>
+      <c r="E1" s="146"/>
+      <c r="F1" s="146"/>
+      <c r="G1" s="146"/>
+      <c r="H1" s="146"/>
+      <c r="I1" s="146"/>
+      <c r="J1" s="146"/>
+      <c r="K1" s="146"/>
     </row>
     <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
@@ -10300,10 +10354,10 @@
       </c>
     </row>
     <row r="33" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D33" s="153" t="s">
+      <c r="D33" s="147" t="s">
         <v>121</v>
       </c>
-      <c r="E33" s="153"/>
+      <c r="E33" s="147"/>
     </row>
     <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="D34" s="70">
@@ -10355,137 +10409,137 @@
     </row>
     <row r="40" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="41" spans="1:11" s="67" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="154" t="s">
+      <c r="A41" s="148" t="s">
         <v>128</v>
       </c>
-      <c r="B41" s="154"/>
-      <c r="C41" s="154"/>
-      <c r="D41" s="154"/>
-      <c r="E41" s="154"/>
-      <c r="F41" s="154"/>
-      <c r="G41" s="154"/>
-      <c r="H41" s="154"/>
-      <c r="I41" s="154"/>
-      <c r="J41" s="154"/>
-      <c r="K41" s="154"/>
+      <c r="B41" s="148"/>
+      <c r="C41" s="148"/>
+      <c r="D41" s="148"/>
+      <c r="E41" s="148"/>
+      <c r="F41" s="148"/>
+      <c r="G41" s="148"/>
+      <c r="H41" s="148"/>
+      <c r="I41" s="148"/>
+      <c r="J41" s="148"/>
+      <c r="K41" s="148"/>
     </row>
     <row r="42" spans="1:11" s="67" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="155" t="s">
+      <c r="A42" s="149" t="s">
         <v>129</v>
       </c>
-      <c r="B42" s="155"/>
-      <c r="C42" s="155"/>
-      <c r="D42" s="155"/>
-      <c r="E42" s="155"/>
-      <c r="F42" s="155"/>
-      <c r="G42" s="155"/>
-      <c r="H42" s="155"/>
-      <c r="I42" s="155"/>
-      <c r="J42" s="155"/>
-      <c r="K42" s="155"/>
+      <c r="B42" s="149"/>
+      <c r="C42" s="149"/>
+      <c r="D42" s="149"/>
+      <c r="E42" s="149"/>
+      <c r="F42" s="149"/>
+      <c r="G42" s="149"/>
+      <c r="H42" s="149"/>
+      <c r="I42" s="149"/>
+      <c r="J42" s="149"/>
+      <c r="K42" s="149"/>
     </row>
     <row r="43" spans="1:11" s="67" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="156" t="s">
+      <c r="A43" s="150" t="s">
         <v>130</v>
       </c>
-      <c r="B43" s="156"/>
-      <c r="C43" s="156"/>
-      <c r="D43" s="156"/>
-      <c r="E43" s="156"/>
-      <c r="F43" s="156"/>
-      <c r="G43" s="156"/>
-      <c r="H43" s="156"/>
-      <c r="I43" s="156"/>
-      <c r="J43" s="156"/>
-      <c r="K43" s="156"/>
+      <c r="B43" s="150"/>
+      <c r="C43" s="150"/>
+      <c r="D43" s="150"/>
+      <c r="E43" s="150"/>
+      <c r="F43" s="150"/>
+      <c r="G43" s="150"/>
+      <c r="H43" s="150"/>
+      <c r="I43" s="150"/>
+      <c r="J43" s="150"/>
+      <c r="K43" s="150"/>
     </row>
     <row r="44" spans="1:11" s="67" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="151" t="s">
+      <c r="A44" s="145" t="s">
         <v>131</v>
       </c>
-      <c r="B44" s="151"/>
-      <c r="C44" s="151"/>
-      <c r="D44" s="151"/>
-      <c r="E44" s="151"/>
-      <c r="F44" s="151"/>
-      <c r="G44" s="151"/>
-      <c r="H44" s="151"/>
-      <c r="I44" s="151"/>
-      <c r="J44" s="151"/>
-      <c r="K44" s="151"/>
+      <c r="B44" s="145"/>
+      <c r="C44" s="145"/>
+      <c r="D44" s="145"/>
+      <c r="E44" s="145"/>
+      <c r="F44" s="145"/>
+      <c r="G44" s="145"/>
+      <c r="H44" s="145"/>
+      <c r="I44" s="145"/>
+      <c r="J44" s="145"/>
+      <c r="K44" s="145"/>
     </row>
     <row r="45" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="46" spans="1:11" ht="15" x14ac:dyDescent="0.25">
-      <c r="A46" s="147" t="s">
+      <c r="A46" s="153" t="s">
         <v>132</v>
       </c>
-      <c r="B46" s="147"/>
-      <c r="C46" s="147"/>
-      <c r="D46" s="147"/>
-      <c r="E46" s="147"/>
-      <c r="F46" s="147"/>
-      <c r="G46" s="147"/>
-      <c r="H46" s="147"/>
-      <c r="I46" s="147"/>
-      <c r="J46" s="147"/>
-      <c r="K46" s="147"/>
+      <c r="B46" s="153"/>
+      <c r="C46" s="153"/>
+      <c r="D46" s="153"/>
+      <c r="E46" s="153"/>
+      <c r="F46" s="153"/>
+      <c r="G46" s="153"/>
+      <c r="H46" s="153"/>
+      <c r="I46" s="153"/>
+      <c r="J46" s="153"/>
+      <c r="K46" s="153"/>
     </row>
     <row r="47" spans="1:11" s="76" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="74" t="s">
         <v>133</v>
       </c>
       <c r="B47" s="75"/>
-      <c r="C47" s="148" t="s">
+      <c r="C47" s="154" t="s">
         <v>134</v>
       </c>
-      <c r="D47" s="148"/>
-      <c r="E47" s="148"/>
-      <c r="F47" s="148"/>
-      <c r="G47" s="148"/>
-      <c r="H47" s="148"/>
-      <c r="I47" s="148"/>
-      <c r="J47" s="148"/>
-      <c r="K47" s="148"/>
+      <c r="D47" s="154"/>
+      <c r="E47" s="154"/>
+      <c r="F47" s="154"/>
+      <c r="G47" s="154"/>
+      <c r="H47" s="154"/>
+      <c r="I47" s="154"/>
+      <c r="J47" s="154"/>
+      <c r="K47" s="154"/>
     </row>
     <row r="48" spans="1:11" s="78" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="149"/>
-      <c r="B48" s="145" t="s">
+      <c r="A48" s="155"/>
+      <c r="B48" s="151" t="s">
         <v>135</v>
       </c>
-      <c r="C48" s="145" t="s">
+      <c r="C48" s="151" t="s">
         <v>136</v>
       </c>
-      <c r="D48" s="145" t="s">
+      <c r="D48" s="151" t="s">
         <v>137</v>
       </c>
-      <c r="E48" s="145" t="s">
+      <c r="E48" s="151" t="s">
         <v>106</v>
       </c>
-      <c r="F48" s="145" t="s">
+      <c r="F48" s="151" t="s">
         <v>138</v>
       </c>
-      <c r="G48" s="145" t="s">
+      <c r="G48" s="151" t="s">
         <v>110</v>
       </c>
-      <c r="H48" s="150" t="s">
+      <c r="H48" s="156" t="s">
         <v>139</v>
       </c>
-      <c r="I48" s="150"/>
-      <c r="J48" s="150"/>
-      <c r="K48" s="150"/>
+      <c r="I48" s="156"/>
+      <c r="J48" s="156"/>
+      <c r="K48" s="156"/>
     </row>
     <row r="49" spans="1:11" s="78" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="149"/>
-      <c r="B49" s="145"/>
-      <c r="C49" s="145"/>
-      <c r="D49" s="145"/>
-      <c r="E49" s="145"/>
-      <c r="F49" s="145"/>
-      <c r="G49" s="145"/>
-      <c r="H49" s="145" t="s">
+      <c r="A49" s="155"/>
+      <c r="B49" s="151"/>
+      <c r="C49" s="151"/>
+      <c r="D49" s="151"/>
+      <c r="E49" s="151"/>
+      <c r="F49" s="151"/>
+      <c r="G49" s="151"/>
+      <c r="H49" s="151" t="s">
         <v>140</v>
       </c>
-      <c r="I49" s="145"/>
+      <c r="I49" s="151"/>
       <c r="J49" s="77" t="s">
         <v>141</v>
       </c>
@@ -10493,7 +10547,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="50" spans="1:11" s="78" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" s="78" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A50" s="79">
         <v>1</v>
       </c>
@@ -10516,158 +10570,284 @@
       <c r="G50" s="82" t="s">
         <v>111</v>
       </c>
-      <c r="H50" s="146"/>
-      <c r="I50" s="146"/>
+      <c r="H50" s="152"/>
+      <c r="I50" s="152"/>
       <c r="J50" s="84"/>
       <c r="K50" s="84" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="51" spans="1:11" s="78" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="79"/>
-      <c r="B51" s="80"/>
-      <c r="C51" s="81"/>
-      <c r="D51" s="82"/>
-      <c r="E51" s="82"/>
-      <c r="F51" s="83" t="e">
+    <row r="51" spans="1:11" s="78" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
+      <c r="A51" s="79">
+        <v>2</v>
+      </c>
+      <c r="B51" s="80" t="s">
+        <v>257</v>
+      </c>
+      <c r="C51" s="81">
+        <v>46127</v>
+      </c>
+      <c r="D51" s="82" t="s">
+        <v>104</v>
+      </c>
+      <c r="E51" s="82" t="s">
+        <v>108</v>
+      </c>
+      <c r="F51" s="83" t="str">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G51" s="82"/>
+        <v>Média</v>
+      </c>
+      <c r="G51" s="82" t="s">
+        <v>111</v>
+      </c>
       <c r="H51" s="85"/>
       <c r="I51" s="86"/>
       <c r="J51" s="84"/>
-      <c r="K51" s="84"/>
-    </row>
-    <row r="52" spans="1:11" s="78" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="79"/>
-      <c r="B52" s="80"/>
-      <c r="C52" s="81"/>
-      <c r="D52" s="82"/>
-      <c r="E52" s="82"/>
-      <c r="F52" s="83" t="e">
+      <c r="K51" s="84" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" s="78" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+      <c r="A52" s="79">
+        <v>3</v>
+      </c>
+      <c r="B52" s="80" t="s">
+        <v>258</v>
+      </c>
+      <c r="C52" s="81">
+        <v>46127</v>
+      </c>
+      <c r="D52" s="82" t="s">
+        <v>103</v>
+      </c>
+      <c r="E52" s="82" t="s">
+        <v>108</v>
+      </c>
+      <c r="F52" s="83" t="str">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G52" s="82"/>
+        <v>Baixa</v>
+      </c>
+      <c r="G52" s="82" t="s">
+        <v>111</v>
+      </c>
       <c r="H52" s="85"/>
       <c r="I52" s="86"/>
       <c r="J52" s="84"/>
-      <c r="K52" s="84"/>
-    </row>
-    <row r="53" spans="1:11" s="78" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="79"/>
-      <c r="B53" s="80"/>
-      <c r="C53" s="81"/>
-      <c r="D53" s="82"/>
-      <c r="E53" s="82"/>
-      <c r="F53" s="83" t="e">
+      <c r="K52" s="84" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" s="78" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
+      <c r="A53" s="79">
+        <v>4</v>
+      </c>
+      <c r="B53" s="80" t="s">
+        <v>259</v>
+      </c>
+      <c r="C53" s="81">
+        <v>46127</v>
+      </c>
+      <c r="D53" s="82" t="s">
+        <v>105</v>
+      </c>
+      <c r="E53" s="82" t="s">
+        <v>109</v>
+      </c>
+      <c r="F53" s="83" t="str">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G53" s="82"/>
+        <v>Alta</v>
+      </c>
+      <c r="G53" s="82" t="s">
+        <v>111</v>
+      </c>
       <c r="H53" s="85"/>
       <c r="I53" s="86"/>
       <c r="J53" s="84"/>
-      <c r="K53" s="84"/>
-    </row>
-    <row r="54" spans="1:11" s="78" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="79"/>
-      <c r="B54" s="80"/>
-      <c r="C54" s="81"/>
-      <c r="D54" s="82"/>
-      <c r="E54" s="82"/>
-      <c r="F54" s="83" t="e">
+      <c r="K53" s="84" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" s="78" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+      <c r="A54" s="79">
+        <v>5</v>
+      </c>
+      <c r="B54" s="80" t="s">
+        <v>260</v>
+      </c>
+      <c r="C54" s="81">
+        <v>46127</v>
+      </c>
+      <c r="D54" s="82" t="s">
+        <v>105</v>
+      </c>
+      <c r="E54" s="82" t="s">
+        <v>109</v>
+      </c>
+      <c r="F54" s="83" t="str">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G54" s="82"/>
+        <v>Alta</v>
+      </c>
+      <c r="G54" s="82" t="s">
+        <v>111</v>
+      </c>
       <c r="H54" s="85"/>
       <c r="I54" s="86"/>
       <c r="J54" s="84"/>
-      <c r="K54" s="84"/>
-    </row>
-    <row r="55" spans="1:11" s="78" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="79"/>
-      <c r="B55" s="80"/>
-      <c r="C55" s="81"/>
-      <c r="D55" s="82"/>
-      <c r="E55" s="82"/>
-      <c r="F55" s="83" t="e">
+      <c r="K54" s="84" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" s="78" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+      <c r="A55" s="79">
+        <v>6</v>
+      </c>
+      <c r="B55" s="80" t="s">
+        <v>261</v>
+      </c>
+      <c r="C55" s="81">
+        <v>46127</v>
+      </c>
+      <c r="D55" s="82" t="s">
+        <v>103</v>
+      </c>
+      <c r="E55" s="82" t="s">
+        <v>108</v>
+      </c>
+      <c r="F55" s="83" t="str">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G55" s="82"/>
+        <v>Baixa</v>
+      </c>
+      <c r="G55" s="82" t="s">
+        <v>111</v>
+      </c>
       <c r="H55" s="85"/>
       <c r="I55" s="86"/>
       <c r="J55" s="84"/>
-      <c r="K55" s="84"/>
-    </row>
-    <row r="56" spans="1:11" s="78" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="79"/>
-      <c r="B56" s="80"/>
-      <c r="C56" s="81"/>
-      <c r="D56" s="82"/>
-      <c r="E56" s="82"/>
-      <c r="F56" s="83" t="e">
+      <c r="K55" s="84" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" s="78" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+      <c r="A56" s="79">
+        <v>7</v>
+      </c>
+      <c r="B56" s="80" t="s">
+        <v>262</v>
+      </c>
+      <c r="C56" s="81">
+        <v>46127</v>
+      </c>
+      <c r="D56" s="82" t="s">
+        <v>104</v>
+      </c>
+      <c r="E56" s="82" t="s">
+        <v>109</v>
+      </c>
+      <c r="F56" s="83" t="str">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G56" s="82"/>
+        <v>Alta</v>
+      </c>
+      <c r="G56" s="82" t="s">
+        <v>111</v>
+      </c>
       <c r="H56" s="85"/>
       <c r="I56" s="86"/>
       <c r="J56" s="84"/>
-      <c r="K56" s="84"/>
-    </row>
-    <row r="57" spans="1:11" s="78" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="79"/>
-      <c r="B57" s="80"/>
-      <c r="C57" s="81"/>
-      <c r="D57" s="82"/>
-      <c r="E57" s="82"/>
-      <c r="F57" s="83" t="e">
+      <c r="K56" s="84" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" s="78" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
+      <c r="A57" s="79">
+        <v>8</v>
+      </c>
+      <c r="B57" s="80" t="s">
+        <v>263</v>
+      </c>
+      <c r="C57" s="81">
+        <v>46127</v>
+      </c>
+      <c r="D57" s="82" t="s">
+        <v>103</v>
+      </c>
+      <c r="E57" s="82" t="s">
+        <v>107</v>
+      </c>
+      <c r="F57" s="83" t="str">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G57" s="82"/>
+        <v>Baixa</v>
+      </c>
+      <c r="G57" s="82" t="s">
+        <v>111</v>
+      </c>
       <c r="H57" s="85"/>
       <c r="I57" s="86"/>
       <c r="J57" s="84"/>
-      <c r="K57" s="84"/>
-    </row>
-    <row r="58" spans="1:11" s="78" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="79"/>
-      <c r="B58" s="80"/>
-      <c r="C58" s="81"/>
-      <c r="D58" s="82"/>
-      <c r="E58" s="82"/>
-      <c r="F58" s="83" t="e">
+      <c r="K57" s="84" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" s="78" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+      <c r="A58" s="79">
+        <v>9</v>
+      </c>
+      <c r="B58" s="80" t="s">
+        <v>264</v>
+      </c>
+      <c r="C58" s="81">
+        <v>46127</v>
+      </c>
+      <c r="D58" s="82" t="s">
+        <v>103</v>
+      </c>
+      <c r="E58" s="82" t="s">
+        <v>109</v>
+      </c>
+      <c r="F58" s="83" t="str">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G58" s="82"/>
+        <v>Média</v>
+      </c>
+      <c r="G58" s="82" t="s">
+        <v>111</v>
+      </c>
       <c r="H58" s="85"/>
       <c r="I58" s="86"/>
       <c r="J58" s="84"/>
-      <c r="K58" s="84"/>
-    </row>
-    <row r="59" spans="1:11" s="78" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="79"/>
-      <c r="B59" s="80"/>
-      <c r="C59" s="81"/>
-      <c r="D59" s="82"/>
-      <c r="E59" s="82"/>
-      <c r="F59" s="83" t="e">
+      <c r="K58" s="84" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" s="78" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+      <c r="A59" s="79">
+        <v>10</v>
+      </c>
+      <c r="B59" s="80" t="s">
+        <v>265</v>
+      </c>
+      <c r="C59" s="81">
+        <v>46127</v>
+      </c>
+      <c r="D59" s="82" t="s">
+        <v>103</v>
+      </c>
+      <c r="E59" s="82" t="s">
+        <v>109</v>
+      </c>
+      <c r="F59" s="83" t="str">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G59" s="82"/>
-      <c r="H59" s="146"/>
-      <c r="I59" s="146"/>
+        <v>Média</v>
+      </c>
+      <c r="G59" s="82" t="s">
+        <v>111</v>
+      </c>
+      <c r="H59" s="152"/>
+      <c r="I59" s="152"/>
       <c r="J59" s="84"/>
-      <c r="K59" s="84"/>
-    </row>
-    <row r="60" spans="1:11" s="78" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K59" s="84" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" s="78" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A60" s="79"/>
       <c r="B60" s="80"/>
       <c r="C60" s="81"/>
@@ -10678,19 +10858,13 @@
         <v>#VALUE!</v>
       </c>
       <c r="G60" s="82"/>
-      <c r="H60" s="146"/>
-      <c r="I60" s="146"/>
+      <c r="H60" s="152"/>
+      <c r="I60" s="152"/>
       <c r="J60" s="84"/>
       <c r="K60" s="84"/>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A42:K42"/>
-    <mergeCell ref="A43:K43"/>
     <mergeCell ref="H49:I49"/>
     <mergeCell ref="H50:I50"/>
     <mergeCell ref="H59:I59"/>
@@ -10705,6 +10879,12 @@
     <mergeCell ref="F48:F49"/>
     <mergeCell ref="G48:G49"/>
     <mergeCell ref="H48:K48"/>
+    <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A43:K43"/>
   </mergeCells>
   <conditionalFormatting sqref="F50:F60">
     <cfRule type="cellIs" dxfId="9" priority="8" stopIfTrue="1" operator="equal">
@@ -10724,7 +10904,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E50:E60 IZ50:IZ60 SV50:SV60 ACR50:ACR60 E65558:E65560 IZ65558:IZ65560 SV65558:SV65560 ACR65558:ACR65560 E65569:E65571 IZ65569:IZ65571 SV65569:SV65571 ACR65569:ACR65571 E65580:E65582 IZ65580:IZ65582 SV65580:SV65582 ACR65580:ACR65582 E65591:E65593 IZ65591:IZ65593 SV65591:SV65593 ACR65591:ACR65593 E131094:E131096 IZ131094:IZ131096 SV131094:SV131096 ACR131094:ACR131096 E131105:E131107 IZ131105:IZ131107 SV131105:SV131107 ACR131105:ACR131107 E131116:E131118 IZ131116:IZ131118 SV131116:SV131118 ACR131116:ACR131118 E131127:E131129 IZ131127:IZ131129 SV131127:SV131129 ACR131127:ACR131129 E196630:E196632 IZ196630:IZ196632 SV196630:SV196632 ACR196630:ACR196632 E196641:E196643 IZ196641:IZ196643 SV196641:SV196643 ACR196641:ACR196643 E196652:E196654 IZ196652:IZ196654 SV196652:SV196654 ACR196652:ACR196654 E196663:E196665 IZ196663:IZ196665 SV196663:SV196665 ACR196663:ACR196665 E262166:E262168 IZ262166:IZ262168 SV262166:SV262168 ACR262166:ACR262168 E262177:E262179 IZ262177:IZ262179 SV262177:SV262179 ACR262177:ACR262179 E262188:E262190 IZ262188:IZ262190 SV262188:SV262190 ACR262188:ACR262190 E262199:E262201 IZ262199:IZ262201 SV262199:SV262201 ACR262199:ACR262201 E327702:E327704 IZ327702:IZ327704 SV327702:SV327704 ACR327702:ACR327704 E327713:E327715 IZ327713:IZ327715 SV327713:SV327715 ACR327713:ACR327715 E327724:E327726 IZ327724:IZ327726 SV327724:SV327726 ACR327724:ACR327726 E327735:E327737 IZ327735:IZ327737 SV327735:SV327737 ACR327735:ACR327737 E393238:E393240 IZ393238:IZ393240 SV393238:SV393240 ACR393238:ACR393240 E393249:E393251 IZ393249:IZ393251 SV393249:SV393251 ACR393249:ACR393251 E393260:E393262 IZ393260:IZ393262 SV393260:SV393262 ACR393260:ACR393262 E393271:E393273 IZ393271:IZ393273 SV393271:SV393273 ACR393271:ACR393273 E458774:E458776 IZ458774:IZ458776 SV458774:SV458776 ACR458774:ACR458776 E458785:E458787 IZ458785:IZ458787 SV458785:SV458787 ACR458785:ACR458787 E458796:E458798 IZ458796:IZ458798 SV458796:SV458798 ACR458796:ACR458798 E458807:E458809 IZ458807:IZ458809 SV458807:SV458809 ACR458807:ACR458809 E524310:E524312 IZ524310:IZ524312 SV524310:SV524312 ACR524310:ACR524312 E524321:E524323 IZ524321:IZ524323 SV524321:SV524323 ACR524321:ACR524323 E524332:E524334 IZ524332:IZ524334 SV524332:SV524334 ACR524332:ACR524334 E524343:E524345 IZ524343:IZ524345 SV524343:SV524345 ACR524343:ACR524345 E589846:E589848 IZ589846:IZ589848 SV589846:SV589848 ACR589846:ACR589848 E589857:E589859 IZ589857:IZ589859 SV589857:SV589859 ACR589857:ACR589859 E589868:E589870 IZ589868:IZ589870 SV589868:SV589870 ACR589868:ACR589870 E589879:E589881 IZ589879:IZ589881 SV589879:SV589881 ACR589879:ACR589881 E655382:E655384 IZ655382:IZ655384 SV655382:SV655384 ACR655382:ACR655384 E655393:E655395 IZ655393:IZ655395 SV655393:SV655395 ACR655393:ACR655395 E655404:E655406 IZ655404:IZ655406 SV655404:SV655406 ACR655404:ACR655406 E655415:E655417 IZ655415:IZ655417 SV655415:SV655417 ACR655415:ACR655417 E720918:E720920 IZ720918:IZ720920 SV720918:SV720920 ACR720918:ACR720920 E720929:E720931 IZ720929:IZ720931 SV720929:SV720931 ACR720929:ACR720931 E720940:E720942 IZ720940:IZ720942 SV720940:SV720942 ACR720940:ACR720942 E720951:E720953 IZ720951:IZ720953 SV720951:SV720953 ACR720951:ACR720953 E786454:E786456 IZ786454:IZ786456 SV786454:SV786456 ACR786454:ACR786456 E786465:E786467 IZ786465:IZ786467 SV786465:SV786467 ACR786465:ACR786467 E786476:E786478 IZ786476:IZ786478 SV786476:SV786478 ACR786476:ACR786478 E786487:E786489 IZ786487:IZ786489 SV786487:SV786489 ACR786487:ACR786489 E851990:E851992 IZ851990:IZ851992 SV851990:SV851992 ACR851990:ACR851992 E852001:E852003 IZ852001:IZ852003 SV852001:SV852003 ACR852001:ACR852003 E852012:E852014 IZ852012:IZ852014 SV852012:SV852014 ACR852012:ACR852014 E852023:E852025 IZ852023:IZ852025 SV852023:SV852025 ACR852023:ACR852025 E917526:E917528 IZ917526:IZ917528 SV917526:SV917528 ACR917526:ACR917528 E917537:E917539 IZ917537:IZ917539 SV917537:SV917539 ACR917537:ACR917539 E917548:E917550 IZ917548:IZ917550 SV917548:SV917550 ACR917548:ACR917550 E917559:E917561 IZ917559:IZ917561 SV917559:SV917561 ACR917559:ACR917561 E983062:E983064 IZ983062:IZ983064 SV983062:SV983064 ACR983062:ACR983064 E983073:E983075 IZ983073:IZ983075 SV983073:SV983075 ACR983073:ACR983075 E983084:E983086 IZ983084:IZ983086 SV983084:SV983086 ACR983084:ACR983086 E983095:E983097 IZ983095:IZ983097 SV983095:SV983097 ACR983095:ACR983097" xr:uid="{00000000-0002-0000-0400-000001000000}">
       <formula1>$D$19:$D$21</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G50:G60 JB50:JB60 SX50:SX60 ACT50:ACT60 G65558:G65560 JB65558:JB65560 SX65558:SX65560 ACT65558:ACT65560 G65569:G65571 JB65569:JB65571 SX65569:SX65571 ACT65569:ACT65571 G65580:G65582 JB65580:JB65582 SX65580:SX65582 ACT65580:ACT65582 G65591:G65593 JB65591:JB65593 SX65591:SX65593 ACT65591:ACT65593 G131094:G131096 JB131094:JB131096 SX131094:SX131096 ACT131094:ACT131096 G131105:G131107 JB131105:JB131107 SX131105:SX131107 ACT131105:ACT131107 G131116:G131118 JB131116:JB131118 SX131116:SX131118 ACT131116:ACT131118 G131127:G131129 JB131127:JB131129 SX131127:SX131129 ACT131127:ACT131129 G196630:G196632 JB196630:JB196632 SX196630:SX196632 ACT196630:ACT196632 G196641:G196643 JB196641:JB196643 SX196641:SX196643 ACT196641:ACT196643 G196652:G196654 JB196652:JB196654 SX196652:SX196654 ACT196652:ACT196654 G196663:G196665 JB196663:JB196665 SX196663:SX196665 ACT196663:ACT196665 G262166:G262168 JB262166:JB262168 SX262166:SX262168 ACT262166:ACT262168 G262177:G262179 JB262177:JB262179 SX262177:SX262179 ACT262177:ACT262179 G262188:G262190 JB262188:JB262190 SX262188:SX262190 ACT262188:ACT262190 G262199:G262201 JB262199:JB262201 SX262199:SX262201 ACT262199:ACT262201 G327702:G327704 JB327702:JB327704 SX327702:SX327704 ACT327702:ACT327704 G327713:G327715 JB327713:JB327715 SX327713:SX327715 ACT327713:ACT327715 G327724:G327726 JB327724:JB327726 SX327724:SX327726 ACT327724:ACT327726 G327735:G327737 JB327735:JB327737 SX327735:SX327737 ACT327735:ACT327737 G393238:G393240 JB393238:JB393240 SX393238:SX393240 ACT393238:ACT393240 G393249:G393251 JB393249:JB393251 SX393249:SX393251 ACT393249:ACT393251 G393260:G393262 JB393260:JB393262 SX393260:SX393262 ACT393260:ACT393262 G393271:G393273 JB393271:JB393273 SX393271:SX393273 ACT393271:ACT393273 G458774:G458776 JB458774:JB458776 SX458774:SX458776 ACT458774:ACT458776 G458785:G458787 JB458785:JB458787 SX458785:SX458787 ACT458785:ACT458787 G458796:G458798 JB458796:JB458798 SX458796:SX458798 ACT458796:ACT458798 G458807:G458809 JB458807:JB458809 SX458807:SX458809 ACT458807:ACT458809 G524310:G524312 JB524310:JB524312 SX524310:SX524312 ACT524310:ACT524312 G524321:G524323 JB524321:JB524323 SX524321:SX524323 ACT524321:ACT524323 G524332:G524334 JB524332:JB524334 SX524332:SX524334 ACT524332:ACT524334 G524343:G524345 JB524343:JB524345 SX524343:SX524345 ACT524343:ACT524345 G589846:G589848 JB589846:JB589848 SX589846:SX589848 ACT589846:ACT589848 G589857:G589859 JB589857:JB589859 SX589857:SX589859 ACT589857:ACT589859 G589868:G589870 JB589868:JB589870 SX589868:SX589870 ACT589868:ACT589870 G589879:G589881 JB589879:JB589881 SX589879:SX589881 ACT589879:ACT589881 G655382:G655384 JB655382:JB655384 SX655382:SX655384 ACT655382:ACT655384 G655393:G655395 JB655393:JB655395 SX655393:SX655395 ACT655393:ACT655395 G655404:G655406 JB655404:JB655406 SX655404:SX655406 ACT655404:ACT655406 G655415:G655417 JB655415:JB655417 SX655415:SX655417 ACT655415:ACT655417 G720918:G720920 JB720918:JB720920 SX720918:SX720920 ACT720918:ACT720920 G720929:G720931 JB720929:JB720931 SX720929:SX720931 ACT720929:ACT720931 G720940:G720942 JB720940:JB720942 SX720940:SX720942 ACT720940:ACT720942 G720951:G720953 JB720951:JB720953 SX720951:SX720953 ACT720951:ACT720953 G786454:G786456 JB786454:JB786456 SX786454:SX786456 ACT786454:ACT786456 G786465:G786467 JB786465:JB786467 SX786465:SX786467 ACT786465:ACT786467 G786476:G786478 JB786476:JB786478 SX786476:SX786478 ACT786476:ACT786478 G786487:G786489 JB786487:JB786489 SX786487:SX786489 ACT786487:ACT786489 G851990:G851992 JB851990:JB851992 SX851990:SX851992 ACT851990:ACT851992 G852001:G852003 JB852001:JB852003 SX852001:SX852003 ACT852001:ACT852003 G852012:G852014 JB852012:JB852014 SX852012:SX852014 ACT852012:ACT852014 G852023:G852025 JB852023:JB852025 SX852023:SX852025 ACT852023:ACT852025 G917526:G917528 JB917526:JB917528 SX917526:SX917528 ACT917526:ACT917528 G917537:G917539 JB917537:JB917539 SX917537:SX917539 ACT917537:ACT917539 G917548:G917550 JB917548:JB917550 SX917548:SX917550 ACT917548:ACT917550 G917559:G917561 JB917559:JB917561 SX917559:SX917561 ACT917559:ACT917561 G983062:G983064 JB983062:JB983064 SX983062:SX983064 ACT983062:ACT983064 G983073:G983075 JB983073:JB983075 SX983073:SX983075 ACT983073:ACT983075 G983084:G983086 JB983084:JB983086 SX983084:SX983086 ACT983084:ACT983086 G983095:G983097 JB983095:JB983097 SX983095:SX983097 ACT983095:ACT983097" xr:uid="{00000000-0002-0000-0400-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ACT983095:ACT983097 JB50:JB60 SX50:SX60 ACT50:ACT60 G65558:G65560 JB65558:JB65560 SX65558:SX65560 ACT65558:ACT65560 G65569:G65571 JB65569:JB65571 SX65569:SX65571 ACT65569:ACT65571 G65580:G65582 JB65580:JB65582 SX65580:SX65582 ACT65580:ACT65582 G65591:G65593 JB65591:JB65593 SX65591:SX65593 ACT65591:ACT65593 G131094:G131096 JB131094:JB131096 SX131094:SX131096 ACT131094:ACT131096 G131105:G131107 JB131105:JB131107 SX131105:SX131107 ACT131105:ACT131107 G131116:G131118 JB131116:JB131118 SX131116:SX131118 ACT131116:ACT131118 G131127:G131129 JB131127:JB131129 SX131127:SX131129 ACT131127:ACT131129 G196630:G196632 JB196630:JB196632 SX196630:SX196632 ACT196630:ACT196632 G196641:G196643 JB196641:JB196643 SX196641:SX196643 ACT196641:ACT196643 G196652:G196654 JB196652:JB196654 SX196652:SX196654 ACT196652:ACT196654 G196663:G196665 JB196663:JB196665 SX196663:SX196665 ACT196663:ACT196665 G262166:G262168 JB262166:JB262168 SX262166:SX262168 ACT262166:ACT262168 G262177:G262179 JB262177:JB262179 SX262177:SX262179 ACT262177:ACT262179 G262188:G262190 JB262188:JB262190 SX262188:SX262190 ACT262188:ACT262190 G262199:G262201 JB262199:JB262201 SX262199:SX262201 ACT262199:ACT262201 G327702:G327704 JB327702:JB327704 SX327702:SX327704 ACT327702:ACT327704 G327713:G327715 JB327713:JB327715 SX327713:SX327715 ACT327713:ACT327715 G327724:G327726 JB327724:JB327726 SX327724:SX327726 ACT327724:ACT327726 G327735:G327737 JB327735:JB327737 SX327735:SX327737 ACT327735:ACT327737 G393238:G393240 JB393238:JB393240 SX393238:SX393240 ACT393238:ACT393240 G393249:G393251 JB393249:JB393251 SX393249:SX393251 ACT393249:ACT393251 G393260:G393262 JB393260:JB393262 SX393260:SX393262 ACT393260:ACT393262 G393271:G393273 JB393271:JB393273 SX393271:SX393273 ACT393271:ACT393273 G458774:G458776 JB458774:JB458776 SX458774:SX458776 ACT458774:ACT458776 G458785:G458787 JB458785:JB458787 SX458785:SX458787 ACT458785:ACT458787 G458796:G458798 JB458796:JB458798 SX458796:SX458798 ACT458796:ACT458798 G458807:G458809 JB458807:JB458809 SX458807:SX458809 ACT458807:ACT458809 G524310:G524312 JB524310:JB524312 SX524310:SX524312 ACT524310:ACT524312 G524321:G524323 JB524321:JB524323 SX524321:SX524323 ACT524321:ACT524323 G524332:G524334 JB524332:JB524334 SX524332:SX524334 ACT524332:ACT524334 G524343:G524345 JB524343:JB524345 SX524343:SX524345 ACT524343:ACT524345 G589846:G589848 JB589846:JB589848 SX589846:SX589848 ACT589846:ACT589848 G589857:G589859 JB589857:JB589859 SX589857:SX589859 ACT589857:ACT589859 G589868:G589870 JB589868:JB589870 SX589868:SX589870 ACT589868:ACT589870 G589879:G589881 JB589879:JB589881 SX589879:SX589881 ACT589879:ACT589881 G655382:G655384 JB655382:JB655384 SX655382:SX655384 ACT655382:ACT655384 G655393:G655395 JB655393:JB655395 SX655393:SX655395 ACT655393:ACT655395 G655404:G655406 JB655404:JB655406 SX655404:SX655406 ACT655404:ACT655406 G655415:G655417 JB655415:JB655417 SX655415:SX655417 ACT655415:ACT655417 G720918:G720920 JB720918:JB720920 SX720918:SX720920 ACT720918:ACT720920 G720929:G720931 JB720929:JB720931 SX720929:SX720931 ACT720929:ACT720931 G720940:G720942 JB720940:JB720942 SX720940:SX720942 ACT720940:ACT720942 G720951:G720953 JB720951:JB720953 SX720951:SX720953 ACT720951:ACT720953 G786454:G786456 JB786454:JB786456 SX786454:SX786456 ACT786454:ACT786456 G786465:G786467 JB786465:JB786467 SX786465:SX786467 ACT786465:ACT786467 G786476:G786478 JB786476:JB786478 SX786476:SX786478 ACT786476:ACT786478 G786487:G786489 JB786487:JB786489 SX786487:SX786489 ACT786487:ACT786489 G851990:G851992 JB851990:JB851992 SX851990:SX851992 ACT851990:ACT851992 G852001:G852003 JB852001:JB852003 SX852001:SX852003 ACT852001:ACT852003 G852012:G852014 JB852012:JB852014 SX852012:SX852014 ACT852012:ACT852014 G852023:G852025 JB852023:JB852025 SX852023:SX852025 ACT852023:ACT852025 G917526:G917528 JB917526:JB917528 SX917526:SX917528 ACT917526:ACT917528 G917537:G917539 JB917537:JB917539 SX917537:SX917539 ACT917537:ACT917539 G917548:G917550 JB917548:JB917550 SX917548:SX917550 ACT917548:ACT917550 G917559:G917561 JB917559:JB917561 SX917559:SX917561 ACT917559:ACT917561 G983062:G983064 JB983062:JB983064 SX983062:SX983064 ACT983062:ACT983064 G983073:G983075 JB983073:JB983075 SX983073:SX983075 ACT983073:ACT983075 G983084:G983086 JB983084:JB983086 SX983084:SX983086 ACT983084:ACT983086 G983095:G983097 JB983095:JB983097 SX983095:SX983097 G50:G60" xr:uid="{00000000-0002-0000-0400-000002000000}">
       <formula1>$D$23:$D$26</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H65554:I65554 JC65554:JD65554 SY65554:SZ65554 ACU65554:ACV65554 H65565:I65565 JC65565:JD65565 SY65565:SZ65565 ACU65565:ACV65565 H65576:I65576 JC65576:JD65576 SY65576:SZ65576 ACU65576:ACV65576 H65587:I65587 JC65587:JD65587 SY65587:SZ65587 ACU65587:ACV65587 H131090:I131090 JC131090:JD131090 SY131090:SZ131090 ACU131090:ACV131090 H131101:I131101 JC131101:JD131101 SY131101:SZ131101 ACU131101:ACV131101 H131112:I131112 JC131112:JD131112 SY131112:SZ131112 ACU131112:ACV131112 H131123:I131123 JC131123:JD131123 SY131123:SZ131123 ACU131123:ACV131123 H196626:I196626 JC196626:JD196626 SY196626:SZ196626 ACU196626:ACV196626 H196637:I196637 JC196637:JD196637 SY196637:SZ196637 ACU196637:ACV196637 H196648:I196648 JC196648:JD196648 SY196648:SZ196648 ACU196648:ACV196648 H196659:I196659 JC196659:JD196659 SY196659:SZ196659 ACU196659:ACV196659 H262162:I262162 JC262162:JD262162 SY262162:SZ262162 ACU262162:ACV262162 H262173:I262173 JC262173:JD262173 SY262173:SZ262173 ACU262173:ACV262173 H262184:I262184 JC262184:JD262184 SY262184:SZ262184 ACU262184:ACV262184 H262195:I262195 JC262195:JD262195 SY262195:SZ262195 ACU262195:ACV262195 H327698:I327698 JC327698:JD327698 SY327698:SZ327698 ACU327698:ACV327698 H327709:I327709 JC327709:JD327709 SY327709:SZ327709 ACU327709:ACV327709 H327720:I327720 JC327720:JD327720 SY327720:SZ327720 ACU327720:ACV327720 H327731:I327731 JC327731:JD327731 SY327731:SZ327731 ACU327731:ACV327731 H393234:I393234 JC393234:JD393234 SY393234:SZ393234 ACU393234:ACV393234 H393245:I393245 JC393245:JD393245 SY393245:SZ393245 ACU393245:ACV393245 H393256:I393256 JC393256:JD393256 SY393256:SZ393256 ACU393256:ACV393256 H393267:I393267 JC393267:JD393267 SY393267:SZ393267 ACU393267:ACV393267 H458770:I458770 JC458770:JD458770 SY458770:SZ458770 ACU458770:ACV458770 H458781:I458781 JC458781:JD458781 SY458781:SZ458781 ACU458781:ACV458781 H458792:I458792 JC458792:JD458792 SY458792:SZ458792 ACU458792:ACV458792 H458803:I458803 JC458803:JD458803 SY458803:SZ458803 ACU458803:ACV458803 H524306:I524306 JC524306:JD524306 SY524306:SZ524306 ACU524306:ACV524306 H524317:I524317 JC524317:JD524317 SY524317:SZ524317 ACU524317:ACV524317 H524328:I524328 JC524328:JD524328 SY524328:SZ524328 ACU524328:ACV524328 H524339:I524339 JC524339:JD524339 SY524339:SZ524339 ACU524339:ACV524339 H589842:I589842 JC589842:JD589842 SY589842:SZ589842 ACU589842:ACV589842 H589853:I589853 JC589853:JD589853 SY589853:SZ589853 ACU589853:ACV589853 H589864:I589864 JC589864:JD589864 SY589864:SZ589864 ACU589864:ACV589864 H589875:I589875 JC589875:JD589875 SY589875:SZ589875 ACU589875:ACV589875 H655378:I655378 JC655378:JD655378 SY655378:SZ655378 ACU655378:ACV655378 H655389:I655389 JC655389:JD655389 SY655389:SZ655389 ACU655389:ACV655389 H655400:I655400 JC655400:JD655400 SY655400:SZ655400 ACU655400:ACV655400 H655411:I655411 JC655411:JD655411 SY655411:SZ655411 ACU655411:ACV655411 H720914:I720914 JC720914:JD720914 SY720914:SZ720914 ACU720914:ACV720914 H720925:I720925 JC720925:JD720925 SY720925:SZ720925 ACU720925:ACV720925 H720936:I720936 JC720936:JD720936 SY720936:SZ720936 ACU720936:ACV720936 H720947:I720947 JC720947:JD720947 SY720947:SZ720947 ACU720947:ACV720947 H786450:I786450 JC786450:JD786450 SY786450:SZ786450 ACU786450:ACV786450 H786461:I786461 JC786461:JD786461 SY786461:SZ786461 ACU786461:ACV786461 H786472:I786472 JC786472:JD786472 SY786472:SZ786472 ACU786472:ACV786472 H786483:I786483 JC786483:JD786483 SY786483:SZ786483 ACU786483:ACV786483 H851986:I851986 JC851986:JD851986 SY851986:SZ851986 ACU851986:ACV851986 H851997:I851997 JC851997:JD851997 SY851997:SZ851997 ACU851997:ACV851997 H852008:I852008 JC852008:JD852008 SY852008:SZ852008 ACU852008:ACV852008 H852019:I852019 JC852019:JD852019 SY852019:SZ852019 ACU852019:ACV852019 H917522:I917522 JC917522:JD917522 SY917522:SZ917522 ACU917522:ACV917522 H917533:I917533 JC917533:JD917533 SY917533:SZ917533 ACU917533:ACV917533 H917544:I917544 JC917544:JD917544 SY917544:SZ917544 ACU917544:ACV917544 H917555:I917555 JC917555:JD917555 SY917555:SZ917555 ACU917555:ACV917555 H983058:I983058 JC983058:JD983058 SY983058:SZ983058 ACU983058:ACV983058 H983069:I983069 JC983069:JD983069 SY983069:SZ983069 ACU983069:ACV983069 H983080:I983080 JC983080:JD983080 SY983080:SZ983080 ACU983080:ACV983080 H983091:I983091 JC983091:JD983091 SY983091:SZ983091 ACU983091:ACV983091" xr:uid="{00000000-0002-0000-0400-000003000000}">
@@ -10755,19 +10935,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="152" t="s">
+      <c r="A1" s="146" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="152"/>
-      <c r="C1" s="152"/>
-      <c r="D1" s="152"/>
-      <c r="E1" s="152"/>
-      <c r="F1" s="152"/>
-      <c r="G1" s="152"/>
-      <c r="H1" s="152"/>
-      <c r="I1" s="152"/>
-      <c r="J1" s="152"/>
-      <c r="K1" s="152"/>
+      <c r="B1" s="146"/>
+      <c r="C1" s="146"/>
+      <c r="D1" s="146"/>
+      <c r="E1" s="146"/>
+      <c r="F1" s="146"/>
+      <c r="G1" s="146"/>
+      <c r="H1" s="146"/>
+      <c r="I1" s="146"/>
+      <c r="J1" s="146"/>
+      <c r="K1" s="146"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="157" t="s">
@@ -10878,7 +11058,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="126" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C6" s="127">
         <v>46113</v>
@@ -10932,7 +11112,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="126" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C8" s="127">
         <v>46141</v>
@@ -11128,7 +11308,7 @@
       <formula>$F5="Ongoing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F14" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"Planejado,Em execução,Entregue,Não planejado"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Inclusao Roteiro de Testes, Inclusao Historia de Usuario e Inclusao Codigo Fonte
</commit_message>
<xml_diff>
--- a/AprovAI/6.Gerenciamento de Projeto/AprovAI - Planejamento e Controle do Projeto.xlsx
+++ b/AprovAI/6.Gerenciamento de Projeto/AprovAI - Planejamento e Controle do Projeto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiag\Downloads\EngenhariaSoftware_AprovAI\AprovAI\AprovAI\6.Gerenciamento de Projeto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C570234F-919A-4612-A104-99A7C6924213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CFBE59E-3C5F-42C0-BE6F-370DF13AF617}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="718" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="718" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Equipe" sheetId="1" r:id="rId1"/>
@@ -6653,18 +6653,6 @@
     <xf numFmtId="164" fontId="22" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="16" fillId="7" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -6673,23 +6661,17 @@
     <xf numFmtId="164" fontId="13" fillId="5" borderId="2" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="33" fillId="15" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6704,6 +6686,24 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="33" fillId="15" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="22" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
@@ -9013,38 +9013,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="144" t="s">
+      <c r="A1" s="140" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="144"/>
-      <c r="C1" s="144"/>
-      <c r="D1" s="144"/>
-      <c r="F1" s="138" t="s">
+      <c r="B1" s="140"/>
+      <c r="C1" s="140"/>
+      <c r="D1" s="140"/>
+      <c r="F1" s="141" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="138"/>
-      <c r="H1" s="138"/>
-      <c r="I1" s="138"/>
-      <c r="J1" s="138"/>
-      <c r="K1" s="138"/>
-      <c r="L1" s="138"/>
+      <c r="G1" s="141"/>
+      <c r="H1" s="141"/>
+      <c r="I1" s="141"/>
+      <c r="J1" s="141"/>
+      <c r="K1" s="141"/>
+      <c r="L1" s="141"/>
     </row>
     <row r="2" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="139" t="s">
+      <c r="A2" s="142" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="139"/>
-      <c r="C2" s="139"/>
-      <c r="D2" s="139"/>
-      <c r="F2" s="140" t="s">
+      <c r="B2" s="142"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="F2" s="143" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="140"/>
-      <c r="H2" s="140"/>
-      <c r="I2" s="140"/>
-      <c r="J2" s="140"/>
-      <c r="K2" s="140"/>
-      <c r="L2" s="140"/>
+      <c r="G2" s="143"/>
+      <c r="H2" s="143"/>
+      <c r="I2" s="143"/>
+      <c r="J2" s="143"/>
+      <c r="K2" s="143"/>
+      <c r="L2" s="143"/>
     </row>
     <row r="3" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
@@ -9065,20 +9065,20 @@
       <c r="G3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="141" t="s">
+      <c r="H3" s="144" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="141"/>
-      <c r="J3" s="141"/>
-      <c r="K3" s="141"/>
-      <c r="L3" s="141"/>
+      <c r="I3" s="144"/>
+      <c r="J3" s="144"/>
+      <c r="K3" s="144"/>
+      <c r="L3" s="144"/>
     </row>
     <row r="4" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="142" t="s">
+      <c r="A4" s="138" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="142"/>
-      <c r="C4" s="142"/>
+      <c r="B4" s="138"/>
+      <c r="C4" s="138"/>
       <c r="D4" s="8" t="s">
         <v>17</v>
       </c>
@@ -9232,10 +9232,10 @@
         <v>225</v>
       </c>
       <c r="H8" s="15">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I8" s="15">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J8" s="15">
         <v>1</v>
@@ -9245,7 +9245,7 @@
       </c>
       <c r="L8" s="16">
         <f t="shared" ref="L8:L18" si="0">SUM(H8:K8)</f>
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
@@ -9321,11 +9321,11 @@
       </c>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="142" t="s">
+      <c r="A11" s="138" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="142"/>
-      <c r="C11" s="142"/>
+      <c r="B11" s="138"/>
+      <c r="C11" s="138"/>
       <c r="D11" s="8">
         <f>SUM(D5:D10)</f>
         <v>10</v>
@@ -9588,11 +9588,11 @@
       <c r="L20" s="21"/>
     </row>
     <row r="21" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="142" t="s">
+      <c r="A21" s="138" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="142"/>
-      <c r="C21" s="142"/>
+      <c r="B21" s="138"/>
+      <c r="C21" s="138"/>
       <c r="D21" s="8">
         <f>SUM(D12:D20)</f>
         <v>82</v>
@@ -9955,11 +9955,11 @@
       </c>
     </row>
     <row r="41" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="142" t="s">
+      <c r="A41" s="138" t="s">
         <v>41</v>
       </c>
-      <c r="B41" s="142"/>
-      <c r="C41" s="142"/>
+      <c r="B41" s="138"/>
+      <c r="C41" s="138"/>
       <c r="D41" s="8">
         <f>SUM(D22:D40)</f>
         <v>130</v>
@@ -10092,9 +10092,9 @@
       </c>
     </row>
     <row r="51" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="143"/>
-      <c r="B51" s="143"/>
-      <c r="C51" s="143"/>
+      <c r="A51" s="139"/>
+      <c r="B51" s="139"/>
+      <c r="C51" s="139"/>
       <c r="D51" s="8">
         <f>SUM(D42:D50)</f>
         <v>85</v>
@@ -10108,16 +10108,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="F1:L1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="F2:L2"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="A4:C4"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A41:C41"/>
     <mergeCell ref="A51:C51"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="F1:L1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="F2:L2"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="A4:C4"/>
   </mergeCells>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="1.1437007874015752" bottom="1.1437007874015752" header="0.75000000000000011" footer="0.75000000000000011"/>
   <pageSetup paperSize="0" fitToWidth="0" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
@@ -10188,19 +10188,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="67" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="146" t="s">
+      <c r="A1" s="152" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="146"/>
-      <c r="C1" s="146"/>
-      <c r="D1" s="146"/>
-      <c r="E1" s="146"/>
-      <c r="F1" s="146"/>
-      <c r="G1" s="146"/>
-      <c r="H1" s="146"/>
-      <c r="I1" s="146"/>
-      <c r="J1" s="146"/>
-      <c r="K1" s="146"/>
+      <c r="B1" s="152"/>
+      <c r="C1" s="152"/>
+      <c r="D1" s="152"/>
+      <c r="E1" s="152"/>
+      <c r="F1" s="152"/>
+      <c r="G1" s="152"/>
+      <c r="H1" s="152"/>
+      <c r="I1" s="152"/>
+      <c r="J1" s="152"/>
+      <c r="K1" s="152"/>
     </row>
     <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
@@ -10354,10 +10354,10 @@
       </c>
     </row>
     <row r="33" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D33" s="147" t="s">
+      <c r="D33" s="153" t="s">
         <v>121</v>
       </c>
-      <c r="E33" s="147"/>
+      <c r="E33" s="153"/>
     </row>
     <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="D34" s="70">
@@ -10409,137 +10409,137 @@
     </row>
     <row r="40" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="41" spans="1:11" s="67" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="148" t="s">
+      <c r="A41" s="154" t="s">
         <v>128</v>
       </c>
-      <c r="B41" s="148"/>
-      <c r="C41" s="148"/>
-      <c r="D41" s="148"/>
-      <c r="E41" s="148"/>
-      <c r="F41" s="148"/>
-      <c r="G41" s="148"/>
-      <c r="H41" s="148"/>
-      <c r="I41" s="148"/>
-      <c r="J41" s="148"/>
-      <c r="K41" s="148"/>
+      <c r="B41" s="154"/>
+      <c r="C41" s="154"/>
+      <c r="D41" s="154"/>
+      <c r="E41" s="154"/>
+      <c r="F41" s="154"/>
+      <c r="G41" s="154"/>
+      <c r="H41" s="154"/>
+      <c r="I41" s="154"/>
+      <c r="J41" s="154"/>
+      <c r="K41" s="154"/>
     </row>
     <row r="42" spans="1:11" s="67" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="149" t="s">
+      <c r="A42" s="155" t="s">
         <v>129</v>
       </c>
-      <c r="B42" s="149"/>
-      <c r="C42" s="149"/>
-      <c r="D42" s="149"/>
-      <c r="E42" s="149"/>
-      <c r="F42" s="149"/>
-      <c r="G42" s="149"/>
-      <c r="H42" s="149"/>
-      <c r="I42" s="149"/>
-      <c r="J42" s="149"/>
-      <c r="K42" s="149"/>
+      <c r="B42" s="155"/>
+      <c r="C42" s="155"/>
+      <c r="D42" s="155"/>
+      <c r="E42" s="155"/>
+      <c r="F42" s="155"/>
+      <c r="G42" s="155"/>
+      <c r="H42" s="155"/>
+      <c r="I42" s="155"/>
+      <c r="J42" s="155"/>
+      <c r="K42" s="155"/>
     </row>
     <row r="43" spans="1:11" s="67" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="150" t="s">
+      <c r="A43" s="156" t="s">
         <v>130</v>
       </c>
-      <c r="B43" s="150"/>
-      <c r="C43" s="150"/>
-      <c r="D43" s="150"/>
-      <c r="E43" s="150"/>
-      <c r="F43" s="150"/>
-      <c r="G43" s="150"/>
-      <c r="H43" s="150"/>
-      <c r="I43" s="150"/>
-      <c r="J43" s="150"/>
-      <c r="K43" s="150"/>
+      <c r="B43" s="156"/>
+      <c r="C43" s="156"/>
+      <c r="D43" s="156"/>
+      <c r="E43" s="156"/>
+      <c r="F43" s="156"/>
+      <c r="G43" s="156"/>
+      <c r="H43" s="156"/>
+      <c r="I43" s="156"/>
+      <c r="J43" s="156"/>
+      <c r="K43" s="156"/>
     </row>
     <row r="44" spans="1:11" s="67" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="145" t="s">
+      <c r="A44" s="151" t="s">
         <v>131</v>
       </c>
-      <c r="B44" s="145"/>
-      <c r="C44" s="145"/>
-      <c r="D44" s="145"/>
-      <c r="E44" s="145"/>
-      <c r="F44" s="145"/>
-      <c r="G44" s="145"/>
-      <c r="H44" s="145"/>
-      <c r="I44" s="145"/>
-      <c r="J44" s="145"/>
-      <c r="K44" s="145"/>
+      <c r="B44" s="151"/>
+      <c r="C44" s="151"/>
+      <c r="D44" s="151"/>
+      <c r="E44" s="151"/>
+      <c r="F44" s="151"/>
+      <c r="G44" s="151"/>
+      <c r="H44" s="151"/>
+      <c r="I44" s="151"/>
+      <c r="J44" s="151"/>
+      <c r="K44" s="151"/>
     </row>
     <row r="45" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="46" spans="1:11" ht="15" x14ac:dyDescent="0.25">
-      <c r="A46" s="153" t="s">
+      <c r="A46" s="147" t="s">
         <v>132</v>
       </c>
-      <c r="B46" s="153"/>
-      <c r="C46" s="153"/>
-      <c r="D46" s="153"/>
-      <c r="E46" s="153"/>
-      <c r="F46" s="153"/>
-      <c r="G46" s="153"/>
-      <c r="H46" s="153"/>
-      <c r="I46" s="153"/>
-      <c r="J46" s="153"/>
-      <c r="K46" s="153"/>
+      <c r="B46" s="147"/>
+      <c r="C46" s="147"/>
+      <c r="D46" s="147"/>
+      <c r="E46" s="147"/>
+      <c r="F46" s="147"/>
+      <c r="G46" s="147"/>
+      <c r="H46" s="147"/>
+      <c r="I46" s="147"/>
+      <c r="J46" s="147"/>
+      <c r="K46" s="147"/>
     </row>
     <row r="47" spans="1:11" s="76" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="74" t="s">
         <v>133</v>
       </c>
       <c r="B47" s="75"/>
-      <c r="C47" s="154" t="s">
+      <c r="C47" s="148" t="s">
         <v>134</v>
       </c>
-      <c r="D47" s="154"/>
-      <c r="E47" s="154"/>
-      <c r="F47" s="154"/>
-      <c r="G47" s="154"/>
-      <c r="H47" s="154"/>
-      <c r="I47" s="154"/>
-      <c r="J47" s="154"/>
-      <c r="K47" s="154"/>
+      <c r="D47" s="148"/>
+      <c r="E47" s="148"/>
+      <c r="F47" s="148"/>
+      <c r="G47" s="148"/>
+      <c r="H47" s="148"/>
+      <c r="I47" s="148"/>
+      <c r="J47" s="148"/>
+      <c r="K47" s="148"/>
     </row>
     <row r="48" spans="1:11" s="78" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="155"/>
-      <c r="B48" s="151" t="s">
+      <c r="A48" s="149"/>
+      <c r="B48" s="145" t="s">
         <v>135</v>
       </c>
-      <c r="C48" s="151" t="s">
+      <c r="C48" s="145" t="s">
         <v>136</v>
       </c>
-      <c r="D48" s="151" t="s">
+      <c r="D48" s="145" t="s">
         <v>137</v>
       </c>
-      <c r="E48" s="151" t="s">
+      <c r="E48" s="145" t="s">
         <v>106</v>
       </c>
-      <c r="F48" s="151" t="s">
+      <c r="F48" s="145" t="s">
         <v>138</v>
       </c>
-      <c r="G48" s="151" t="s">
+      <c r="G48" s="145" t="s">
         <v>110</v>
       </c>
-      <c r="H48" s="156" t="s">
+      <c r="H48" s="150" t="s">
         <v>139</v>
       </c>
-      <c r="I48" s="156"/>
-      <c r="J48" s="156"/>
-      <c r="K48" s="156"/>
+      <c r="I48" s="150"/>
+      <c r="J48" s="150"/>
+      <c r="K48" s="150"/>
     </row>
     <row r="49" spans="1:11" s="78" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="155"/>
-      <c r="B49" s="151"/>
-      <c r="C49" s="151"/>
-      <c r="D49" s="151"/>
-      <c r="E49" s="151"/>
-      <c r="F49" s="151"/>
-      <c r="G49" s="151"/>
-      <c r="H49" s="151" t="s">
+      <c r="A49" s="149"/>
+      <c r="B49" s="145"/>
+      <c r="C49" s="145"/>
+      <c r="D49" s="145"/>
+      <c r="E49" s="145"/>
+      <c r="F49" s="145"/>
+      <c r="G49" s="145"/>
+      <c r="H49" s="145" t="s">
         <v>140</v>
       </c>
-      <c r="I49" s="151"/>
+      <c r="I49" s="145"/>
       <c r="J49" s="77" t="s">
         <v>141</v>
       </c>
@@ -10570,8 +10570,8 @@
       <c r="G50" s="82" t="s">
         <v>111</v>
       </c>
-      <c r="H50" s="152"/>
-      <c r="I50" s="152"/>
+      <c r="H50" s="146"/>
+      <c r="I50" s="146"/>
       <c r="J50" s="84"/>
       <c r="K50" s="84" t="s">
         <v>254</v>
@@ -10840,8 +10840,8 @@
       <c r="G59" s="82" t="s">
         <v>111</v>
       </c>
-      <c r="H59" s="152"/>
-      <c r="I59" s="152"/>
+      <c r="H59" s="146"/>
+      <c r="I59" s="146"/>
       <c r="J59" s="84"/>
       <c r="K59" s="84" t="s">
         <v>274</v>
@@ -10858,13 +10858,19 @@
         <v>#VALUE!</v>
       </c>
       <c r="G60" s="82"/>
-      <c r="H60" s="152"/>
-      <c r="I60" s="152"/>
+      <c r="H60" s="146"/>
+      <c r="I60" s="146"/>
       <c r="J60" s="84"/>
       <c r="K60" s="84"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A43:K43"/>
     <mergeCell ref="H49:I49"/>
     <mergeCell ref="H50:I50"/>
     <mergeCell ref="H59:I59"/>
@@ -10879,12 +10885,6 @@
     <mergeCell ref="F48:F49"/>
     <mergeCell ref="G48:G49"/>
     <mergeCell ref="H48:K48"/>
-    <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A42:K42"/>
-    <mergeCell ref="A43:K43"/>
   </mergeCells>
   <conditionalFormatting sqref="F50:F60">
     <cfRule type="cellIs" dxfId="9" priority="8" stopIfTrue="1" operator="equal">
@@ -10935,19 +10935,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="146" t="s">
+      <c r="A1" s="152" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="146"/>
-      <c r="C1" s="146"/>
-      <c r="D1" s="146"/>
-      <c r="E1" s="146"/>
-      <c r="F1" s="146"/>
-      <c r="G1" s="146"/>
-      <c r="H1" s="146"/>
-      <c r="I1" s="146"/>
-      <c r="J1" s="146"/>
-      <c r="K1" s="146"/>
+      <c r="B1" s="152"/>
+      <c r="C1" s="152"/>
+      <c r="D1" s="152"/>
+      <c r="E1" s="152"/>
+      <c r="F1" s="152"/>
+      <c r="G1" s="152"/>
+      <c r="H1" s="152"/>
+      <c r="I1" s="152"/>
+      <c r="J1" s="152"/>
+      <c r="K1" s="152"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="157" t="s">
@@ -11308,7 +11308,7 @@
       <formula>$F5="Ongoing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F14" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"Planejado,Em execução,Entregue,Não planejado"</formula1>
     </dataValidation>

</xml_diff>